<commit_message>
Generate tear sheet Jun 2026
</commit_message>
<xml_diff>
--- a/output/Tear_Sheet_Apr2026.xlsx
+++ b/output/Tear_Sheet_Apr2026.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="117">
   <si>
     <t>Date</t>
   </si>
   <si>
-    <t>VAMI</t>
+    <t>Green Renewable Storage Energy Market Participation and Trading</t>
   </si>
   <si>
     <t>Jul 2022</t>
@@ -161,7 +161,10 @@
     <t>Apr 2026</t>
   </si>
   <si>
-    <t>Return (%)</t>
+    <t>Fund Return (%)</t>
+  </si>
+  <si>
+    <t>iShares MSCI Australia ETF</t>
   </si>
   <si>
     <t>April 2026</t>
@@ -354,6 +357,9 @@
   </si>
   <si>
     <t>Year Return</t>
+  </si>
+  <si>
+    <t>EWA</t>
   </si>
   <si>
     <t>NOTE: This publication has been prepared on behalf of and issued by Green Exchange Pty Ltd (ACN 654 125 247) holding AFSL 559619. This is for educational purposes only. This is not an offer to deal in any financial product. This information might contain unsolicited general information only, without regard to any investor's individual objectives, financial situation or needs. It is not specific advice for any particular investor. Before making any decision about the information provided, you must consider the appropriateness of the information in this document, having regard to your objectives, financial situation and needs and consult your adviser. This may not be passed on to anyone but the addressee. Past performance of financial products is no assurance of future performance.</t>
@@ -1016,6 +1022,323 @@
                 </c:pt>
                 <c:pt idx="46">
                   <c:v>2284.52</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>iShares MSCI Australia ETF</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="15875">
+              <a:solidFill>
+                <a:srgbClr val="9E9E9E"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>_data!$G$2:$G$48</c:f>
+              <c:strCache>
+                <c:ptCount val="47"/>
+                <c:pt idx="0">
+                  <c:v>Jul 2022</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Jul 2022</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Aug 2022</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Sep 2022</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Oct 2022</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Nov 2022</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Dec 2022</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Jan 2023</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Feb 2023</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Mar 2023</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Apr 2023</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>May 2023</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jun 2023</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Jul 2023</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Aug 2023</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Sep 2023</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>Oct 2023</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Nov 2023</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Dec 2023</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Jan 2024</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Feb 2024</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Mar 2024</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Apr 2024</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>May 2024</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>Jun 2024</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>Jul 2024</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>Aug 2024</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>Sep 2024</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>Oct 2024</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>Nov 2024</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>Dec 2024</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>Jan 2025</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>Feb 2025</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>Mar 2025</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>Apr 2025</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>May 2025</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>Jun 2025</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>Jul 2025</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>Aug 2025</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>Sep 2025</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>Oct 2025</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>Nov 2025</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>Dec 2025</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>_data!$H$2:$H$48</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="47"/>
+                <c:pt idx="0">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1105.22</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1064.88</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>953.58</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1007.04</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1151.39</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1080.43</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1231.05</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1133</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1135.97</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1145.88</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1082.99</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1116.66</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1178.42</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1120.41</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1085.09</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1046.25</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1132.51</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1227.86</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1215.73</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1231.17</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1269.26</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1201.32</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>1268.75</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1257.42</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1312.64</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1357.24</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1422.29</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1329.96</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1386.62</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1251.79</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>1312.9</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>1279.83</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1250.48</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>1316.1</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>1376.92</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>1404.13</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>1409.38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>1466.8</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>1462.46</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>1450.01</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>1400.17</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>1418.59</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>1528.78</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>1657.69</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>1529.33</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>1624.64</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2031,10 +2354,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2047,8 +2370,14 @@
       <c r="E1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="G1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2061,8 +2390,14 @@
       <c r="E2">
         <v>5.74</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2075,8 +2410,14 @@
       <c r="E3">
         <v>3.29</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="G3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1105.22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2089,8 +2430,14 @@
       <c r="E4">
         <v>2.62</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="G4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>1064.88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2103,8 +2450,14 @@
       <c r="E5">
         <v>2.7</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="G5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>953.58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2117,8 +2470,14 @@
       <c r="E6">
         <v>1.66</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="G6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>1007.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -2131,8 +2490,14 @@
       <c r="E7">
         <v>1.12</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="G7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7">
+        <v>1151.39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -2145,8 +2510,14 @@
       <c r="E8">
         <v>1.01</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="G8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8">
+        <v>1080.43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2159,8 +2530,14 @@
       <c r="E9">
         <v>1.08</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="G9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9">
+        <v>1231.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2173,8 +2550,14 @@
       <c r="E10">
         <v>2.23</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="G10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -2187,8 +2570,14 @@
       <c r="E11">
         <v>2.46</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>1135.97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2201,8 +2590,14 @@
       <c r="E12">
         <v>4.31</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="G12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12">
+        <v>1145.88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2215,8 +2610,14 @@
       <c r="E13">
         <v>1.64</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="G13" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13">
+        <v>1082.99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -2229,8 +2630,14 @@
       <c r="E14">
         <v>1.49</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14">
+        <v>1116.66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2243,8 +2650,14 @@
       <c r="E15">
         <v>2.04</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="G15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15">
+        <v>1178.42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2257,8 +2670,14 @@
       <c r="E16">
         <v>0.96</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16">
+        <v>1120.41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2271,8 +2690,14 @@
       <c r="E17">
         <v>0.26</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="G17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17">
+        <v>1085.09</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2285,8 +2710,14 @@
       <c r="E18">
         <v>1.8</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="G18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18">
+        <v>1046.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2299,8 +2730,14 @@
       <c r="E19">
         <v>0.89</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="G19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19">
+        <v>1132.51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2313,8 +2750,14 @@
       <c r="E20">
         <v>2.02</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="G20" t="s">
+        <v>19</v>
+      </c>
+      <c r="H20">
+        <v>1227.86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2327,8 +2770,14 @@
       <c r="E21">
         <v>1.24</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="G21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21">
+        <v>1215.73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2341,8 +2790,14 @@
       <c r="E22">
         <v>1.12</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="G22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22">
+        <v>1231.17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -2355,8 +2810,14 @@
       <c r="E23">
         <v>1.47</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="G23" t="s">
+        <v>22</v>
+      </c>
+      <c r="H23">
+        <v>1269.26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -2369,8 +2830,14 @@
       <c r="E24">
         <v>8.98</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="G24" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24">
+        <v>1201.32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -2383,8 +2850,14 @@
       <c r="E25">
         <v>1.16</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="G25" t="s">
+        <v>24</v>
+      </c>
+      <c r="H25">
+        <v>1268.75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -2397,8 +2870,14 @@
       <c r="E26">
         <v>0.24</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="G26" t="s">
+        <v>25</v>
+      </c>
+      <c r="H26">
+        <v>1257.42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -2411,8 +2890,14 @@
       <c r="E27">
         <v>2.58</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="G27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27">
+        <v>1312.64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -2425,8 +2910,14 @@
       <c r="E28">
         <v>0.35</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="G28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28">
+        <v>1357.24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -2439,8 +2930,14 @@
       <c r="E29">
         <v>1.94</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="G29" t="s">
+        <v>28</v>
+      </c>
+      <c r="H29">
+        <v>1422.29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -2453,8 +2950,14 @@
       <c r="E30">
         <v>4.99</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="G30" t="s">
+        <v>29</v>
+      </c>
+      <c r="H30">
+        <v>1329.96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -2467,8 +2970,14 @@
       <c r="E31">
         <v>1.22</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="G31" t="s">
+        <v>30</v>
+      </c>
+      <c r="H31">
+        <v>1386.62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -2481,8 +2990,14 @@
       <c r="E32">
         <v>0.24</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="G32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H32">
+        <v>1251.79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2495,8 +3010,14 @@
       <c r="E33">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="G33" t="s">
+        <v>32</v>
+      </c>
+      <c r="H33">
+        <v>1312.9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -2509,8 +3030,14 @@
       <c r="E34">
         <v>1.9</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="G34" t="s">
+        <v>33</v>
+      </c>
+      <c r="H34">
+        <v>1279.83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -2523,8 +3050,14 @@
       <c r="E35">
         <v>0.98</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="G35" t="s">
+        <v>34</v>
+      </c>
+      <c r="H35">
+        <v>1250.48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -2537,8 +3070,14 @@
       <c r="E36">
         <v>1.48</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="G36" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36">
+        <v>1316.1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -2551,8 +3090,14 @@
       <c r="E37">
         <v>4.24</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="G37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H37">
+        <v>1376.92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -2565,8 +3110,14 @@
       <c r="E38">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="G38" t="s">
+        <v>37</v>
+      </c>
+      <c r="H38">
+        <v>1404.13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -2579,8 +3130,14 @@
       <c r="E39">
         <v>2.41</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="G39" t="s">
+        <v>38</v>
+      </c>
+      <c r="H39">
+        <v>1409.38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -2593,8 +3150,14 @@
       <c r="E40">
         <v>1.46</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="G40" t="s">
+        <v>39</v>
+      </c>
+      <c r="H40">
+        <v>1466.8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -2607,8 +3170,14 @@
       <c r="E41">
         <v>1.76</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="G41" t="s">
+        <v>40</v>
+      </c>
+      <c r="H41">
+        <v>1462.46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -2621,8 +3190,14 @@
       <c r="E42">
         <v>-0.54</v>
       </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="G42" t="s">
+        <v>41</v>
+      </c>
+      <c r="H42">
+        <v>1450.01</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -2635,8 +3210,14 @@
       <c r="E43">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="G43" t="s">
+        <v>42</v>
+      </c>
+      <c r="H43">
+        <v>1400.17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -2649,8 +3230,14 @@
       <c r="E44">
         <v>1.54</v>
       </c>
-    </row>
-    <row r="45" spans="1:5">
+      <c r="G44" t="s">
+        <v>43</v>
+      </c>
+      <c r="H44">
+        <v>1418.59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2663,8 +3250,14 @@
       <c r="E45">
         <v>1.46</v>
       </c>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="G45" t="s">
+        <v>44</v>
+      </c>
+      <c r="H45">
+        <v>1528.78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -2677,8 +3270,14 @@
       <c r="E46">
         <v>0.65</v>
       </c>
-    </row>
-    <row r="47" spans="1:5">
+      <c r="G46" t="s">
+        <v>45</v>
+      </c>
+      <c r="H46">
+        <v>1657.69</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -2691,13 +3290,25 @@
       <c r="E47">
         <v>0.6899999999999999</v>
       </c>
-    </row>
-    <row r="48" spans="1:5">
+      <c r="G47" t="s">
+        <v>46</v>
+      </c>
+      <c r="H47">
+        <v>1529.33</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" t="s">
         <v>47</v>
       </c>
       <c r="B48">
         <v>2284.52</v>
+      </c>
+      <c r="G48" t="s">
+        <v>47</v>
+      </c>
+      <c r="H48">
+        <v>1624.64</v>
       </c>
     </row>
   </sheetData>
@@ -2723,7 +3334,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="14" customHeight="1">
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2742,7 +3353,7 @@
     </row>
     <row r="2" spans="1:17" ht="26" customHeight="1">
       <c r="B2" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2761,7 +3372,7 @@
     </row>
     <row r="3" spans="1:17" ht="26" customHeight="1">
       <c r="B3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2800,7 +3411,7 @@
     <row r="5" spans="1:17" ht="8" customHeight="1"/>
     <row r="6" spans="1:17" ht="17" customHeight="1">
       <c r="B6" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2810,7 +3421,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -2821,7 +3432,7 @@
     </row>
     <row r="7" spans="1:17">
       <c r="B7" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2831,7 +3442,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
@@ -2842,7 +3453,7 @@
     </row>
     <row r="8" spans="1:17">
       <c r="B8" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -2861,7 +3472,7 @@
     </row>
     <row r="9" spans="1:17">
       <c r="B9" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -2880,7 +3491,7 @@
     </row>
     <row r="10" spans="1:17">
       <c r="B10" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -2899,7 +3510,7 @@
     </row>
     <row r="11" spans="1:17">
       <c r="B11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -2935,7 +3546,7 @@
     </row>
     <row r="13" spans="1:17" ht="17" customHeight="1">
       <c r="B13" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -2945,7 +3556,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
@@ -2956,7 +3567,7 @@
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
       <c r="B14" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -2966,14 +3577,14 @@
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
       <c r="O14" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P14" s="8"/>
     </row>
@@ -2987,20 +3598,20 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
       <c r="N15" s="9"/>
       <c r="O15" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P15" s="9"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
       <c r="B16" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -3010,20 +3621,20 @@
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
       <c r="J16" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
       <c r="O16" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P16" s="8"/>
     </row>
     <row r="17" spans="2:16" ht="26" customHeight="1">
       <c r="B17" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -3033,20 +3644,20 @@
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
       <c r="J17" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K17" s="11"/>
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
       <c r="O17" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P17" s="9"/>
     </row>
     <row r="18" spans="2:16" ht="10" customHeight="1">
       <c r="B18" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
@@ -3065,7 +3676,7 @@
     </row>
     <row r="19" spans="2:16" ht="17" customHeight="1">
       <c r="B19" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
@@ -3075,7 +3686,7 @@
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
       <c r="J19" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
@@ -3086,7 +3697,7 @@
     </row>
     <row r="20" spans="2:16">
       <c r="B20" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -3096,14 +3707,14 @@
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
       <c r="J20" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K20" s="12"/>
       <c r="L20" s="12"/>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
       <c r="O20" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P20" s="13"/>
     </row>
@@ -3117,20 +3728,20 @@
       <c r="H21" s="10"/>
       <c r="I21" s="10"/>
       <c r="J21" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
       <c r="O21" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="P21" s="13"/>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -3140,20 +3751,20 @@
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
       <c r="J22" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K22" s="12"/>
       <c r="L22" s="12"/>
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
       <c r="O22" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="P22" s="13"/>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
@@ -3163,14 +3774,14 @@
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
       <c r="J23" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K23" s="12"/>
       <c r="L23" s="12"/>
       <c r="M23" s="12"/>
       <c r="N23" s="12"/>
       <c r="O23" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P23" s="13"/>
     </row>
@@ -3184,14 +3795,14 @@
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
       <c r="J24" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K24" s="12"/>
       <c r="L24" s="12"/>
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
       <c r="O24" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P24" s="13"/>
     </row>
@@ -3214,7 +3825,7 @@
     </row>
     <row r="26" spans="2:16" ht="17" customHeight="1">
       <c r="B26" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -3224,7 +3835,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
@@ -3243,14 +3854,14 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
       <c r="M27" s="12"/>
       <c r="N27" s="12"/>
       <c r="O27" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P27" s="14"/>
     </row>
@@ -3264,14 +3875,14 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K28" s="12"/>
       <c r="L28" s="12"/>
       <c r="M28" s="12"/>
       <c r="N28" s="12"/>
       <c r="O28" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P28" s="14"/>
     </row>
@@ -3285,14 +3896,14 @@
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K29" s="12"/>
       <c r="L29" s="12"/>
       <c r="M29" s="12"/>
       <c r="N29" s="12"/>
       <c r="O29" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P29" s="14"/>
     </row>
@@ -3306,14 +3917,14 @@
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K30" s="12"/>
       <c r="L30" s="12"/>
       <c r="M30" s="12"/>
       <c r="N30" s="12"/>
       <c r="O30" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P30" s="14"/>
     </row>
@@ -3473,7 +4084,7 @@
     <row r="40" spans="2:16" ht="10" customHeight="1"/>
     <row r="41" spans="2:16" ht="17" customHeight="1">
       <c r="B41" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -3680,7 +4291,7 @@
     <row r="53" spans="2:16" ht="8" customHeight="1"/>
     <row r="54" spans="2:16" ht="17" customHeight="1">
       <c r="B54" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
@@ -3700,45 +4311,47 @@
     <row r="55" spans="2:16" ht="16" customHeight="1">
       <c r="B55" s="15"/>
       <c r="C55" s="15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G55" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H55" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I55" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J55" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L55" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M55" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N55" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O55" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="P55" s="15"/>
+        <v>113</v>
+      </c>
+      <c r="P55" s="15" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="56" spans="2:16" ht="14" customHeight="1">
       <c r="B56" s="16">
@@ -3767,7 +4380,9 @@
       <c r="O56" s="19">
         <v>4.41</v>
       </c>
-      <c r="P56" s="19"/>
+      <c r="P56" s="17">
+        <v>14.52</v>
+      </c>
     </row>
     <row r="57" spans="2:16" ht="14" customHeight="1">
       <c r="B57" s="20">
@@ -3812,7 +4427,9 @@
       <c r="O57" s="23">
         <v>15.99</v>
       </c>
-      <c r="P57" s="23"/>
+      <c r="P57" s="21">
+        <v>13.33</v>
+      </c>
     </row>
     <row r="58" spans="2:16" ht="14" customHeight="1">
       <c r="B58" s="16">
@@ -3857,7 +4474,9 @@
       <c r="O58" s="19">
         <v>30.6</v>
       </c>
-      <c r="P58" s="19"/>
+      <c r="P58" s="17">
+        <v>1.95</v>
+      </c>
     </row>
     <row r="59" spans="2:16" ht="14" customHeight="1">
       <c r="B59" s="20">
@@ -3902,7 +4521,9 @@
       <c r="O59" s="23">
         <v>22.07</v>
       </c>
-      <c r="P59" s="23"/>
+      <c r="P59" s="21">
+        <v>13.65</v>
+      </c>
     </row>
     <row r="60" spans="2:16" ht="14" customHeight="1">
       <c r="B60" s="16">
@@ -3935,12 +4556,14 @@
       <c r="O60" s="19">
         <v>18.33</v>
       </c>
-      <c r="P60" s="19"/>
+      <c r="P60" s="17">
+        <v>8.039999999999999</v>
+      </c>
     </row>
     <row r="61" spans="2:16" ht="6" customHeight="1"/>
     <row r="62" spans="2:16" ht="40" customHeight="1">
       <c r="B62" s="24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C62" s="24"/>
       <c r="D62" s="24"/>
@@ -3959,7 +4582,7 @@
     </row>
     <row r="63" spans="2:16" ht="16" customHeight="1">
       <c r="B63" s="10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="10"/>
@@ -3977,7 +4600,7 @@
       <c r="P63" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="107">
+  <mergeCells count="101">
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="J1:P1"/>
     <mergeCell ref="B2:P2"/>
@@ -4077,12 +4700,6 @@
     <mergeCell ref="B51:P51"/>
     <mergeCell ref="B52:P52"/>
     <mergeCell ref="B54:P54"/>
-    <mergeCell ref="O55:P55"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="O57:P57"/>
-    <mergeCell ref="O58:P58"/>
-    <mergeCell ref="O59:P59"/>
-    <mergeCell ref="O60:P60"/>
     <mergeCell ref="B62:P62"/>
     <mergeCell ref="B63:P63"/>
   </mergeCells>

</xml_diff>

<commit_message>
Tear Sheet first tab, Data second tab; unhide data sheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Tear_Sheet_Apr2026.xlsx
+++ b/output/Tear_Sheet_Apr2026.xlsx
@@ -7,8 +7,8 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="_data" sheetId="1" r:id="rId1"/>
-    <sheet name="Tear Sheet" sheetId="2" r:id="rId2"/>
+    <sheet name="Tear Sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -729,7 +729,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>_data!$A$2:$A$48</c:f>
+              <c:f>Data!$A$2:$A$48</c:f>
               <c:strCache>
                 <c:ptCount val="47"/>
                 <c:pt idx="0">
@@ -878,7 +878,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>_data!$B$2:$B$48</c:f>
+              <c:f>Data!$B$2:$B$48</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="47"/>
@@ -1046,7 +1046,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>_data!$G$2:$G$48</c:f>
+              <c:f>Data!$G$2:$G$48</c:f>
               <c:strCache>
                 <c:ptCount val="47"/>
                 <c:pt idx="0">
@@ -1195,7 +1195,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>_data!$H$2:$H$48</c:f>
+              <c:f>Data!$H$2:$H$48</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="47"/>
@@ -1523,7 +1523,7 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>_data!$D$2:$D$47</c:f>
+              <c:f>Data!$D$2:$D$47</c:f>
               <c:strCache>
                 <c:ptCount val="46"/>
                 <c:pt idx="0">
@@ -1669,7 +1669,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>_data!$E$2:$E$47</c:f>
+              <c:f>Data!$E$2:$E$47</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="46"/>
@@ -2354,970 +2354,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H48"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
-        <v>1000</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>5.74</v>
-      </c>
-      <c r="G2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1057.4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>3.29</v>
-      </c>
-      <c r="G3" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>1105.22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1092.19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4">
-        <v>2.62</v>
-      </c>
-      <c r="G4" t="s">
-        <v>3</v>
-      </c>
-      <c r="H4">
-        <v>1064.88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>1120.8</v>
-      </c>
-      <c r="D5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>2.7</v>
-      </c>
-      <c r="G5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>953.58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>1151.07</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>1.66</v>
-      </c>
-      <c r="G6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6">
-        <v>1007.04</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>1170.17</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7">
-        <v>1.12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7">
-        <v>1151.39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>1183.28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8">
-        <v>1.01</v>
-      </c>
-      <c r="G8" t="s">
-        <v>7</v>
-      </c>
-      <c r="H8">
-        <v>1080.43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>1195.23</v>
-      </c>
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9">
-        <v>1.08</v>
-      </c>
-      <c r="G9" t="s">
-        <v>8</v>
-      </c>
-      <c r="H9">
-        <v>1231.05</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>1208.14</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10">
-        <v>2.23</v>
-      </c>
-      <c r="G10" t="s">
-        <v>9</v>
-      </c>
-      <c r="H10">
-        <v>1133</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>1235.08</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11">
-        <v>2.46</v>
-      </c>
-      <c r="G11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H11">
-        <v>1135.97</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>1265.46</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12">
-        <v>4.31</v>
-      </c>
-      <c r="G12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H12">
-        <v>1145.88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>1320</v>
-      </c>
-      <c r="D13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13">
-        <v>1.64</v>
-      </c>
-      <c r="G13" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13">
-        <v>1082.99</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>1341.65</v>
-      </c>
-      <c r="D14" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14">
-        <v>1.49</v>
-      </c>
-      <c r="G14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14">
-        <v>1116.66</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>1361.64</v>
-      </c>
-      <c r="D15" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15">
-        <v>2.04</v>
-      </c>
-      <c r="G15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15">
-        <v>1178.42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>1389.42</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16">
-        <v>0.96</v>
-      </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16">
-        <v>1120.41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>1402.76</v>
-      </c>
-      <c r="D17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17">
-        <v>0.26</v>
-      </c>
-      <c r="G17" t="s">
-        <v>16</v>
-      </c>
-      <c r="H17">
-        <v>1085.09</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>1406.41</v>
-      </c>
-      <c r="D18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E18">
-        <v>1.8</v>
-      </c>
-      <c r="G18" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18">
-        <v>1046.25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>1431.72</v>
-      </c>
-      <c r="D19" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19">
-        <v>0.89</v>
-      </c>
-      <c r="G19" t="s">
-        <v>18</v>
-      </c>
-      <c r="H19">
-        <v>1132.51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>1444.46</v>
-      </c>
-      <c r="D20" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20">
-        <v>2.02</v>
-      </c>
-      <c r="G20" t="s">
-        <v>19</v>
-      </c>
-      <c r="H20">
-        <v>1227.86</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>1473.64</v>
-      </c>
-      <c r="D21" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21">
-        <v>1.24</v>
-      </c>
-      <c r="G21" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21">
-        <v>1215.73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>1491.92</v>
-      </c>
-      <c r="D22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22">
-        <v>1.12</v>
-      </c>
-      <c r="G22" t="s">
-        <v>21</v>
-      </c>
-      <c r="H22">
-        <v>1231.17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>1508.62</v>
-      </c>
-      <c r="D23" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23">
-        <v>1.47</v>
-      </c>
-      <c r="G23" t="s">
-        <v>22</v>
-      </c>
-      <c r="H23">
-        <v>1269.26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>1530.8</v>
-      </c>
-      <c r="D24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24">
-        <v>8.98</v>
-      </c>
-      <c r="G24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H24">
-        <v>1201.32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>1668.27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25">
-        <v>1.16</v>
-      </c>
-      <c r="G25" t="s">
-        <v>24</v>
-      </c>
-      <c r="H25">
-        <v>1268.75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>1687.62</v>
-      </c>
-      <c r="D26" t="s">
-        <v>26</v>
-      </c>
-      <c r="E26">
-        <v>0.24</v>
-      </c>
-      <c r="G26" t="s">
-        <v>25</v>
-      </c>
-      <c r="H26">
-        <v>1257.42</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>1691.67</v>
-      </c>
-      <c r="D27" t="s">
-        <v>27</v>
-      </c>
-      <c r="E27">
-        <v>2.58</v>
-      </c>
-      <c r="G27" t="s">
-        <v>26</v>
-      </c>
-      <c r="H27">
-        <v>1312.64</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>1735.31</v>
-      </c>
-      <c r="D28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28">
-        <v>0.35</v>
-      </c>
-      <c r="G28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H28">
-        <v>1357.24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>1741.39</v>
-      </c>
-      <c r="D29" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29">
-        <v>1.94</v>
-      </c>
-      <c r="G29" t="s">
-        <v>28</v>
-      </c>
-      <c r="H29">
-        <v>1422.29</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30">
-        <v>1775.17</v>
-      </c>
-      <c r="D30" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30">
-        <v>4.99</v>
-      </c>
-      <c r="G30" t="s">
-        <v>29</v>
-      </c>
-      <c r="H30">
-        <v>1329.96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>1863.75</v>
-      </c>
-      <c r="D31" t="s">
-        <v>31</v>
-      </c>
-      <c r="E31">
-        <v>1.22</v>
-      </c>
-      <c r="G31" t="s">
-        <v>30</v>
-      </c>
-      <c r="H31">
-        <v>1386.62</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32">
-        <v>1886.49</v>
-      </c>
-      <c r="D32" t="s">
-        <v>32</v>
-      </c>
-      <c r="E32">
-        <v>0.24</v>
-      </c>
-      <c r="G32" t="s">
-        <v>31</v>
-      </c>
-      <c r="H32">
-        <v>1251.79</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33">
-        <v>1891.02</v>
-      </c>
-      <c r="D33" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33">
-        <v>0.6</v>
-      </c>
-      <c r="G33" t="s">
-        <v>32</v>
-      </c>
-      <c r="H33">
-        <v>1312.9</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34">
-        <v>1902.36</v>
-      </c>
-      <c r="D34" t="s">
-        <v>34</v>
-      </c>
-      <c r="E34">
-        <v>1.9</v>
-      </c>
-      <c r="G34" t="s">
-        <v>33</v>
-      </c>
-      <c r="H34">
-        <v>1279.83</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35">
-        <v>1938.51</v>
-      </c>
-      <c r="D35" t="s">
-        <v>35</v>
-      </c>
-      <c r="E35">
-        <v>0.98</v>
-      </c>
-      <c r="G35" t="s">
-        <v>34</v>
-      </c>
-      <c r="H35">
-        <v>1250.48</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36">
-        <v>1957.51</v>
-      </c>
-      <c r="D36" t="s">
-        <v>36</v>
-      </c>
-      <c r="E36">
-        <v>1.48</v>
-      </c>
-      <c r="G36" t="s">
-        <v>35</v>
-      </c>
-      <c r="H36">
-        <v>1316.1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37">
-        <v>1986.48</v>
-      </c>
-      <c r="D37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E37">
-        <v>4.24</v>
-      </c>
-      <c r="G37" t="s">
-        <v>36</v>
-      </c>
-      <c r="H37">
-        <v>1376.92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38">
-        <v>2070.7</v>
-      </c>
-      <c r="D38" t="s">
-        <v>38</v>
-      </c>
-      <c r="E38">
-        <v>0.1</v>
-      </c>
-      <c r="G38" t="s">
-        <v>37</v>
-      </c>
-      <c r="H38">
-        <v>1404.13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39">
-        <v>2072.77</v>
-      </c>
-      <c r="D39" t="s">
-        <v>39</v>
-      </c>
-      <c r="E39">
-        <v>2.41</v>
-      </c>
-      <c r="G39" t="s">
-        <v>38</v>
-      </c>
-      <c r="H39">
-        <v>1409.38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>2122.73</v>
-      </c>
-      <c r="D40" t="s">
-        <v>40</v>
-      </c>
-      <c r="E40">
-        <v>1.46</v>
-      </c>
-      <c r="G40" t="s">
-        <v>39</v>
-      </c>
-      <c r="H40">
-        <v>1466.8</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" t="s">
-        <v>40</v>
-      </c>
-      <c r="B41">
-        <v>2153.72</v>
-      </c>
-      <c r="D41" t="s">
-        <v>41</v>
-      </c>
-      <c r="E41">
-        <v>1.76</v>
-      </c>
-      <c r="G41" t="s">
-        <v>40</v>
-      </c>
-      <c r="H41">
-        <v>1462.46</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" t="s">
-        <v>41</v>
-      </c>
-      <c r="B42">
-        <v>2191.63</v>
-      </c>
-      <c r="D42" t="s">
-        <v>42</v>
-      </c>
-      <c r="E42">
-        <v>-0.54</v>
-      </c>
-      <c r="G42" t="s">
-        <v>41</v>
-      </c>
-      <c r="H42">
-        <v>1450.01</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" t="s">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>2179.79</v>
-      </c>
-      <c r="D43" t="s">
-        <v>43</v>
-      </c>
-      <c r="E43">
-        <v>0.38</v>
-      </c>
-      <c r="G43" t="s">
-        <v>42</v>
-      </c>
-      <c r="H43">
-        <v>1400.17</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>2188.07</v>
-      </c>
-      <c r="D44" t="s">
-        <v>44</v>
-      </c>
-      <c r="E44">
-        <v>1.54</v>
-      </c>
-      <c r="G44" t="s">
-        <v>43</v>
-      </c>
-      <c r="H44">
-        <v>1418.59</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45">
-        <v>2221.77</v>
-      </c>
-      <c r="D45" t="s">
-        <v>45</v>
-      </c>
-      <c r="E45">
-        <v>1.46</v>
-      </c>
-      <c r="G45" t="s">
-        <v>44</v>
-      </c>
-      <c r="H45">
-        <v>1528.78</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" t="s">
-        <v>45</v>
-      </c>
-      <c r="B46">
-        <v>2254.21</v>
-      </c>
-      <c r="D46" t="s">
-        <v>46</v>
-      </c>
-      <c r="E46">
-        <v>0.65</v>
-      </c>
-      <c r="G46" t="s">
-        <v>45</v>
-      </c>
-      <c r="H46">
-        <v>1657.69</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47">
-        <v>2268.86</v>
-      </c>
-      <c r="D47" t="s">
-        <v>47</v>
-      </c>
-      <c r="E47">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="G47" t="s">
-        <v>46</v>
-      </c>
-      <c r="H47">
-        <v>1529.33</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" t="s">
-        <v>47</v>
-      </c>
-      <c r="B48">
-        <v>2284.52</v>
-      </c>
-      <c r="G48" t="s">
-        <v>47</v>
-      </c>
-      <c r="H48">
-        <v>1624.64</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4707,4 +3743,968 @@
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>5.74</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1057.4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>3.29</v>
+      </c>
+      <c r="G3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1105.22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1092.19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>2.62</v>
+      </c>
+      <c r="G4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>1064.88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1120.8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>2.7</v>
+      </c>
+      <c r="G5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>953.58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1151.07</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>1.66</v>
+      </c>
+      <c r="G6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6">
+        <v>1007.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1170.17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7">
+        <v>1.12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7">
+        <v>1151.39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1183.28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>1.01</v>
+      </c>
+      <c r="G8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8">
+        <v>1080.43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>1195.23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9">
+        <v>1.08</v>
+      </c>
+      <c r="G9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9">
+        <v>1231.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>1208.14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10">
+        <v>2.23</v>
+      </c>
+      <c r="G10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>1235.08</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11">
+        <v>2.46</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>1135.97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>1265.46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12">
+        <v>4.31</v>
+      </c>
+      <c r="G12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12">
+        <v>1145.88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>1320</v>
+      </c>
+      <c r="D13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13">
+        <v>1.64</v>
+      </c>
+      <c r="G13" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13">
+        <v>1082.99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>1341.65</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14">
+        <v>1.49</v>
+      </c>
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14">
+        <v>1116.66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>1361.64</v>
+      </c>
+      <c r="D15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15">
+        <v>2.04</v>
+      </c>
+      <c r="G15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15">
+        <v>1178.42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>1389.42</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16">
+        <v>0.96</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16">
+        <v>1120.41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>1402.76</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17">
+        <v>0.26</v>
+      </c>
+      <c r="G17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17">
+        <v>1085.09</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>1406.41</v>
+      </c>
+      <c r="D18" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18">
+        <v>1.8</v>
+      </c>
+      <c r="G18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18">
+        <v>1046.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>1431.72</v>
+      </c>
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19">
+        <v>0.89</v>
+      </c>
+      <c r="G19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19">
+        <v>1132.51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>1444.46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20">
+        <v>2.02</v>
+      </c>
+      <c r="G20" t="s">
+        <v>19</v>
+      </c>
+      <c r="H20">
+        <v>1227.86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>1473.64</v>
+      </c>
+      <c r="D21" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21">
+        <v>1.24</v>
+      </c>
+      <c r="G21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21">
+        <v>1215.73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>1491.92</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22">
+        <v>1.12</v>
+      </c>
+      <c r="G22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22">
+        <v>1231.17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>1508.62</v>
+      </c>
+      <c r="D23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E23">
+        <v>1.47</v>
+      </c>
+      <c r="G23" t="s">
+        <v>22</v>
+      </c>
+      <c r="H23">
+        <v>1269.26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>1530.8</v>
+      </c>
+      <c r="D24" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24">
+        <v>8.98</v>
+      </c>
+      <c r="G24" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24">
+        <v>1201.32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>1668.27</v>
+      </c>
+      <c r="D25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25">
+        <v>1.16</v>
+      </c>
+      <c r="G25" t="s">
+        <v>24</v>
+      </c>
+      <c r="H25">
+        <v>1268.75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>1687.62</v>
+      </c>
+      <c r="D26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26">
+        <v>0.24</v>
+      </c>
+      <c r="G26" t="s">
+        <v>25</v>
+      </c>
+      <c r="H26">
+        <v>1257.42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>1691.67</v>
+      </c>
+      <c r="D27" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27">
+        <v>2.58</v>
+      </c>
+      <c r="G27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27">
+        <v>1312.64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>1735.31</v>
+      </c>
+      <c r="D28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28">
+        <v>0.35</v>
+      </c>
+      <c r="G28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28">
+        <v>1357.24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>1741.39</v>
+      </c>
+      <c r="D29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29">
+        <v>1.94</v>
+      </c>
+      <c r="G29" t="s">
+        <v>28</v>
+      </c>
+      <c r="H29">
+        <v>1422.29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>1775.17</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="E30">
+        <v>4.99</v>
+      </c>
+      <c r="G30" t="s">
+        <v>29</v>
+      </c>
+      <c r="H30">
+        <v>1329.96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>1863.75</v>
+      </c>
+      <c r="D31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31">
+        <v>1.22</v>
+      </c>
+      <c r="G31" t="s">
+        <v>30</v>
+      </c>
+      <c r="H31">
+        <v>1386.62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>1886.49</v>
+      </c>
+      <c r="D32" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32">
+        <v>0.24</v>
+      </c>
+      <c r="G32" t="s">
+        <v>31</v>
+      </c>
+      <c r="H32">
+        <v>1251.79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>1891.02</v>
+      </c>
+      <c r="D33" t="s">
+        <v>33</v>
+      </c>
+      <c r="E33">
+        <v>0.6</v>
+      </c>
+      <c r="G33" t="s">
+        <v>32</v>
+      </c>
+      <c r="H33">
+        <v>1312.9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>1902.36</v>
+      </c>
+      <c r="D34" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34">
+        <v>1.9</v>
+      </c>
+      <c r="G34" t="s">
+        <v>33</v>
+      </c>
+      <c r="H34">
+        <v>1279.83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>1938.51</v>
+      </c>
+      <c r="D35" t="s">
+        <v>35</v>
+      </c>
+      <c r="E35">
+        <v>0.98</v>
+      </c>
+      <c r="G35" t="s">
+        <v>34</v>
+      </c>
+      <c r="H35">
+        <v>1250.48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>1957.51</v>
+      </c>
+      <c r="D36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E36">
+        <v>1.48</v>
+      </c>
+      <c r="G36" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36">
+        <v>1316.1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>1986.48</v>
+      </c>
+      <c r="D37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37">
+        <v>4.24</v>
+      </c>
+      <c r="G37" t="s">
+        <v>36</v>
+      </c>
+      <c r="H37">
+        <v>1376.92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>2070.7</v>
+      </c>
+      <c r="D38" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38">
+        <v>0.1</v>
+      </c>
+      <c r="G38" t="s">
+        <v>37</v>
+      </c>
+      <c r="H38">
+        <v>1404.13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>2072.77</v>
+      </c>
+      <c r="D39" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39">
+        <v>2.41</v>
+      </c>
+      <c r="G39" t="s">
+        <v>38</v>
+      </c>
+      <c r="H39">
+        <v>1409.38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>2122.73</v>
+      </c>
+      <c r="D40" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40">
+        <v>1.46</v>
+      </c>
+      <c r="G40" t="s">
+        <v>39</v>
+      </c>
+      <c r="H40">
+        <v>1466.8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>2153.72</v>
+      </c>
+      <c r="D41" t="s">
+        <v>41</v>
+      </c>
+      <c r="E41">
+        <v>1.76</v>
+      </c>
+      <c r="G41" t="s">
+        <v>40</v>
+      </c>
+      <c r="H41">
+        <v>1462.46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>2191.63</v>
+      </c>
+      <c r="D42" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42">
+        <v>-0.54</v>
+      </c>
+      <c r="G42" t="s">
+        <v>41</v>
+      </c>
+      <c r="H42">
+        <v>1450.01</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>2179.79</v>
+      </c>
+      <c r="D43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43">
+        <v>0.38</v>
+      </c>
+      <c r="G43" t="s">
+        <v>42</v>
+      </c>
+      <c r="H43">
+        <v>1400.17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>2188.07</v>
+      </c>
+      <c r="D44" t="s">
+        <v>44</v>
+      </c>
+      <c r="E44">
+        <v>1.54</v>
+      </c>
+      <c r="G44" t="s">
+        <v>43</v>
+      </c>
+      <c r="H44">
+        <v>1418.59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>2221.77</v>
+      </c>
+      <c r="D45" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45">
+        <v>1.46</v>
+      </c>
+      <c r="G45" t="s">
+        <v>44</v>
+      </c>
+      <c r="H45">
+        <v>1528.78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>2254.21</v>
+      </c>
+      <c r="D46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E46">
+        <v>0.65</v>
+      </c>
+      <c r="G46" t="s">
+        <v>45</v>
+      </c>
+      <c r="H46">
+        <v>1657.69</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>2268.86</v>
+      </c>
+      <c r="D47" t="s">
+        <v>47</v>
+      </c>
+      <c r="E47">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G47" t="s">
+        <v>46</v>
+      </c>
+      <c r="H47">
+        <v>1529.33</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>2284.52</v>
+      </c>
+      <c r="G48" t="s">
+        <v>47</v>
+      </c>
+      <c r="H48">
+        <v>1624.64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove text wrap from Strategy Description
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Tear_Sheet_Apr2026.xlsx
+++ b/output/Tear_Sheet_Apr2026.xlsx
@@ -613,7 +613,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -641,7 +641,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -681,9 +681,6 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1983,7 +1980,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="46"/>
                 <c:pt idx="0">
-                  <c:v>10.5216</c:v>
+                  <c:v>10.5217</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-3.65</c:v>
@@ -2031,7 +2028,7 @@
                   <c:v>-3.5797</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>8.244999999999999</c:v>
+                  <c:v>8.244899999999999</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>8.418699999999999</c:v>
@@ -3926,23 +3923,23 @@
       <c r="P62" s="23"/>
     </row>
     <row r="63" spans="2:16" ht="16" customHeight="1">
-      <c r="B63" s="24" t="s">
+      <c r="B63" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C63" s="24"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
-      <c r="G63" s="24"/>
-      <c r="H63" s="24"/>
-      <c r="I63" s="24"/>
-      <c r="J63" s="24"/>
-      <c r="K63" s="24"/>
-      <c r="L63" s="24"/>
-      <c r="M63" s="24"/>
-      <c r="N63" s="24"/>
-      <c r="O63" s="24"/>
-      <c r="P63" s="24"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="10"/>
+      <c r="H63" s="10"/>
+      <c r="I63" s="10"/>
+      <c r="J63" s="10"/>
+      <c r="K63" s="10"/>
+      <c r="L63" s="10"/>
+      <c r="M63" s="10"/>
+      <c r="N63" s="10"/>
+      <c r="O63" s="10"/>
+      <c r="P63" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="101">
@@ -4108,7 +4105,7 @@
         <v>2</v>
       </c>
       <c r="K2">
-        <v>10.5216</v>
+        <v>10.5217</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -4524,7 +4521,7 @@
         <v>18</v>
       </c>
       <c r="K18">
-        <v>8.244999999999999</v>
+        <v>8.244899999999999</v>
       </c>
     </row>
     <row r="19" spans="1:11">

</xml_diff>

<commit_message>
Regenerate Apr 2026 tear sheet from Beats data source
</commit_message>
<xml_diff>
--- a/output/Tear_Sheet_Apr2026.xlsx
+++ b/output/Tear_Sheet_Apr2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="111">
   <si>
     <t>Date</t>
   </si>
@@ -23,24 +23,6 @@
     <t>Green Renewable Storage Energy Market Participation and Trading</t>
   </si>
   <si>
-    <t>Jul 2022</t>
-  </si>
-  <si>
-    <t>Aug 2022</t>
-  </si>
-  <si>
-    <t>Sep 2022</t>
-  </si>
-  <si>
-    <t>Oct 2022</t>
-  </si>
-  <si>
-    <t>Nov 2022</t>
-  </si>
-  <si>
-    <t>Dec 2022</t>
-  </si>
-  <si>
     <t>Jan 2023</t>
   </si>
   <si>
@@ -215,10 +197,10 @@
     <t>Year To Date</t>
   </si>
   <si>
-    <t>2.82%</t>
-  </si>
-  <si>
-    <t>4.41%</t>
+    <t>2.80%</t>
+  </si>
+  <si>
+    <t>4.39%</t>
   </si>
   <si>
     <t>Deployment of strategic Battery assets across Eastern Australia. The Energy landscape</t>
@@ -233,10 +215,10 @@
     <t>in Australia presents an Investment opportunity in BESS. This offers multiple revenue</t>
   </si>
   <si>
-    <t>128.45%</t>
-  </si>
-  <si>
-    <t>4.24%</t>
+    <t>157.27%</t>
+  </si>
+  <si>
+    <t>8.77%</t>
   </si>
   <si>
     <t>streams across the entire value chain. Installation of hardware with a 10+ year lifespan</t>
@@ -299,19 +281,19 @@
     <t xml:space="preserve">  Sharpe Ratio</t>
   </si>
   <si>
-    <t>4.17</t>
+    <t>5.05</t>
   </si>
   <si>
     <t xml:space="preserve">  Winning Months (%)</t>
   </si>
   <si>
-    <t>97.83%</t>
+    <t>100.00%</t>
   </si>
   <si>
     <t xml:space="preserve">  Alpha Annualized</t>
   </si>
   <si>
-    <t>24.05%</t>
+    <t>32.77%</t>
   </si>
   <si>
     <t>MONTHLY RETURNS</t>
@@ -375,7 +357,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -498,13 +480,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FFC62828"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="6.5"/>
       <color rgb="FF757575"/>
       <name val="Calibri"/>
@@ -613,7 +588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -673,13 +648,10 @@
     <xf numFmtId="164" fontId="14" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="12" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -718,148 +690,130 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$48</c:f>
+              <c:f>Data!$A$2:$A$42</c:f>
               <c:strCache>
-                <c:ptCount val="47"/>
+                <c:ptCount val="41"/>
                 <c:pt idx="0">
-                  <c:v>Jul 2022</c:v>
+                  <c:v>Jan 2023</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Jul 2022</c:v>
+                  <c:v>Jan 2023</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Aug 2022</c:v>
+                  <c:v>Feb 2023</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Sep 2022</c:v>
+                  <c:v>Mar 2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Oct 2022</c:v>
+                  <c:v>Apr 2023</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Nov 2022</c:v>
+                  <c:v>May 2023</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Dec 2022</c:v>
+                  <c:v>Jun 2023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Jan 2023</c:v>
+                  <c:v>Jul 2023</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Feb 2023</c:v>
+                  <c:v>Aug 2023</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Mar 2023</c:v>
+                  <c:v>Sep 2023</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Apr 2023</c:v>
+                  <c:v>Oct 2023</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>May 2023</c:v>
+                  <c:v>Nov 2023</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Jun 2023</c:v>
+                  <c:v>Dec 2023</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Jul 2023</c:v>
+                  <c:v>Jan 2024</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Aug 2023</c:v>
+                  <c:v>Feb 2024</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>Sep 2023</c:v>
+                  <c:v>Mar 2024</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Oct 2023</c:v>
+                  <c:v>Apr 2024</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>Nov 2023</c:v>
+                  <c:v>May 2024</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>Dec 2023</c:v>
+                  <c:v>Jun 2024</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>Jan 2024</c:v>
+                  <c:v>Jul 2024</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>Feb 2024</c:v>
+                  <c:v>Aug 2024</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>Mar 2024</c:v>
+                  <c:v>Sep 2024</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>Apr 2024</c:v>
+                  <c:v>Oct 2024</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>May 2024</c:v>
+                  <c:v>Nov 2024</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>Jun 2024</c:v>
+                  <c:v>Dec 2024</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>Jul 2024</c:v>
+                  <c:v>Jan 2025</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>Aug 2024</c:v>
+                  <c:v>Feb 2025</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>Sep 2024</c:v>
+                  <c:v>Mar 2025</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>Oct 2024</c:v>
+                  <c:v>Apr 2025</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>Nov 2024</c:v>
+                  <c:v>May 2025</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>Dec 2024</c:v>
+                  <c:v>Jun 2025</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>Jan 2025</c:v>
+                  <c:v>Jul 2025</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>Feb 2025</c:v>
+                  <c:v>Aug 2025</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>Mar 2025</c:v>
+                  <c:v>Sep 2025</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>Apr 2025</c:v>
+                  <c:v>Oct 2025</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>May 2025</c:v>
+                  <c:v>Nov 2025</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>Jun 2025</c:v>
+                  <c:v>Dec 2025</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>Jul 2025</c:v>
+                  <c:v>Jan 2026</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>Aug 2025</c:v>
+                  <c:v>Feb 2026</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>Sep 2025</c:v>
+                  <c:v>Mar 2026</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>Oct 2025</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>Nov 2025</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>Dec 2025</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>Jan 2026</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>Feb 2026</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>Mar 2026</c:v>
-                </c:pt>
-                <c:pt idx="46">
                   <c:v>Apr 2026</c:v>
                 </c:pt>
               </c:strCache>
@@ -867,150 +821,132 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$B$2:$B$48</c:f>
+              <c:f>Data!$B$2:$B$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="47"/>
+                <c:ptCount val="41"/>
                 <c:pt idx="0">
                   <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1057.4</c:v>
+                  <c:v>1010.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1092.19</c:v>
+                  <c:v>1021.01</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1120.8</c:v>
+                  <c:v>1043.78</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1151.07</c:v>
+                  <c:v>1060.16</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1170.17</c:v>
+                  <c:v>1105.86</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1183.28</c:v>
+                  <c:v>1123.99</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1195.23</c:v>
+                  <c:v>1140.74</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1208.14</c:v>
+                  <c:v>1164.01</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1235.08</c:v>
+                  <c:v>1183.34</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1265.46</c:v>
+                  <c:v>1196.59</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1320</c:v>
+                  <c:v>1218.13</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1341.65</c:v>
+                  <c:v>1234.94</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1361.64</c:v>
+                  <c:v>1259.88</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1389.42</c:v>
+                  <c:v>1297.43</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1402.76</c:v>
+                  <c:v>1311.96</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1406.41</c:v>
+                  <c:v>1331.24</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1431.72</c:v>
+                  <c:v>1450.79</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1444.46</c:v>
+                  <c:v>1481.84</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1473.64</c:v>
+                  <c:v>1520.66</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1491.92</c:v>
+                  <c:v>1604.3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1508.62</c:v>
+                  <c:v>1628.84</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1530.8</c:v>
+                  <c:v>1660.44</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1668.27</c:v>
+                  <c:v>1783.48</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1687.62</c:v>
+                  <c:v>1849.29</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1691.67</c:v>
+                  <c:v>1887.76</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1735.31</c:v>
+                  <c:v>1921.17</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1741.39</c:v>
+                  <c:v>1957.67</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1775.17</c:v>
+                  <c:v>1998.2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1863.75</c:v>
+                  <c:v>2056.14</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1886.49</c:v>
+                  <c:v>2215.29</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1891.02</c:v>
+                  <c:v>2250.07</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1902.36</c:v>
+                  <c:v>2290.8</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1938.51</c:v>
+                  <c:v>2324.24</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1957.51</c:v>
+                  <c:v>2365.15</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1986.48</c:v>
+                  <c:v>2420.26</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>2070.7</c:v>
+                  <c:v>2464.55</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>2072.77</c:v>
+                  <c:v>2502.5</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>2122.73</c:v>
+                  <c:v>2538.54</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>2153.72</c:v>
+                  <c:v>2555.04</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>2191.63</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>2179.79</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>2188.07</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>2221.77</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>2254.21</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>2268.86</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>2284.52</c:v>
+                  <c:v>2572.67</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1035,148 +971,130 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$G$2:$G$48</c:f>
+              <c:f>Data!$G$2:$G$42</c:f>
               <c:strCache>
-                <c:ptCount val="47"/>
+                <c:ptCount val="41"/>
                 <c:pt idx="0">
-                  <c:v>Jul 2022</c:v>
+                  <c:v>Jan 2023</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Jul 2022</c:v>
+                  <c:v>Jan 2023</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Aug 2022</c:v>
+                  <c:v>Feb 2023</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Sep 2022</c:v>
+                  <c:v>Mar 2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Oct 2022</c:v>
+                  <c:v>Apr 2023</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Nov 2022</c:v>
+                  <c:v>May 2023</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Dec 2022</c:v>
+                  <c:v>Jun 2023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Jan 2023</c:v>
+                  <c:v>Jul 2023</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Feb 2023</c:v>
+                  <c:v>Aug 2023</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Mar 2023</c:v>
+                  <c:v>Sep 2023</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Apr 2023</c:v>
+                  <c:v>Oct 2023</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>May 2023</c:v>
+                  <c:v>Nov 2023</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Jun 2023</c:v>
+                  <c:v>Dec 2023</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Jul 2023</c:v>
+                  <c:v>Jan 2024</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Aug 2023</c:v>
+                  <c:v>Feb 2024</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>Sep 2023</c:v>
+                  <c:v>Mar 2024</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Oct 2023</c:v>
+                  <c:v>Apr 2024</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>Nov 2023</c:v>
+                  <c:v>May 2024</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>Dec 2023</c:v>
+                  <c:v>Jun 2024</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>Jan 2024</c:v>
+                  <c:v>Jul 2024</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>Feb 2024</c:v>
+                  <c:v>Aug 2024</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>Mar 2024</c:v>
+                  <c:v>Sep 2024</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>Apr 2024</c:v>
+                  <c:v>Oct 2024</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>May 2024</c:v>
+                  <c:v>Nov 2024</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>Jun 2024</c:v>
+                  <c:v>Dec 2024</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>Jul 2024</c:v>
+                  <c:v>Jan 2025</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>Aug 2024</c:v>
+                  <c:v>Feb 2025</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>Sep 2024</c:v>
+                  <c:v>Mar 2025</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>Oct 2024</c:v>
+                  <c:v>Apr 2025</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>Nov 2024</c:v>
+                  <c:v>May 2025</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>Dec 2024</c:v>
+                  <c:v>Jun 2025</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>Jan 2025</c:v>
+                  <c:v>Jul 2025</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>Feb 2025</c:v>
+                  <c:v>Aug 2025</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>Mar 2025</c:v>
+                  <c:v>Sep 2025</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>Apr 2025</c:v>
+                  <c:v>Oct 2025</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>May 2025</c:v>
+                  <c:v>Nov 2025</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>Jun 2025</c:v>
+                  <c:v>Dec 2025</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>Jul 2025</c:v>
+                  <c:v>Jan 2026</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>Aug 2025</c:v>
+                  <c:v>Feb 2026</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>Sep 2025</c:v>
+                  <c:v>Mar 2026</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>Oct 2025</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>Nov 2025</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>Dec 2025</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>Jan 2026</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>Feb 2026</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>Mar 2026</c:v>
-                </c:pt>
-                <c:pt idx="46">
                   <c:v>Apr 2026</c:v>
                 </c:pt>
               </c:strCache>
@@ -1184,150 +1102,132 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$H$2:$H$48</c:f>
+              <c:f>Data!$H$2:$H$42</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="47"/>
+                <c:ptCount val="41"/>
                 <c:pt idx="0">
                   <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1105.22</c:v>
+                  <c:v>1139.41</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1064.88</c:v>
+                  <c:v>1048.66</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>953.58</c:v>
+                  <c:v>1051.41</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1007.04</c:v>
+                  <c:v>1060.58</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1151.39</c:v>
+                  <c:v>1002.37</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1080.43</c:v>
+                  <c:v>1033.53</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1231.05</c:v>
+                  <c:v>1090.7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1133</c:v>
+                  <c:v>1037</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1135.97</c:v>
+                  <c:v>1004.32</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1145.88</c:v>
+                  <c:v>968.37</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1082.99</c:v>
+                  <c:v>1048.21</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1116.66</c:v>
+                  <c:v>1136.45</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1178.42</c:v>
+                  <c:v>1125.23</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1120.41</c:v>
+                  <c:v>1139.52</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1085.09</c:v>
+                  <c:v>1174.77</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1046.25</c:v>
+                  <c:v>1111.89</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1132.51</c:v>
+                  <c:v>1174.3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1227.86</c:v>
+                  <c:v>1163.82</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1215.73</c:v>
+                  <c:v>1214.93</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1231.17</c:v>
+                  <c:v>1256.2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1269.26</c:v>
+                  <c:v>1316.41</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1201.32</c:v>
+                  <c:v>1230.95</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1268.75</c:v>
+                  <c:v>1283.39</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1257.42</c:v>
+                  <c:v>1158.6</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1312.64</c:v>
+                  <c:v>1215.17</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1357.24</c:v>
+                  <c:v>1184.55</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1422.29</c:v>
+                  <c:v>1157.4</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1329.96</c:v>
+                  <c:v>1218.13</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1386.62</c:v>
+                  <c:v>1274.42</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>1251.79</c:v>
+                  <c:v>1299.6</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1312.9</c:v>
+                  <c:v>1304.46</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1279.83</c:v>
+                  <c:v>1357.61</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>1250.48</c:v>
+                  <c:v>1353.59</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1316.1</c:v>
+                  <c:v>1342.06</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1376.92</c:v>
+                  <c:v>1295.94</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1404.13</c:v>
+                  <c:v>1312.99</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>1409.38</c:v>
+                  <c:v>1414.97</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>1466.8</c:v>
+                  <c:v>1534.29</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>1462.46</c:v>
+                  <c:v>1415.48</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>1450.01</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>1400.17</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>1418.59</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>1528.78</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>1657.69</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>1529.33</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>1624.64</c:v>
+                  <c:v>1503.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1512,145 +1412,127 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$D$2:$D$47</c:f>
+              <c:f>Data!$D$2:$D$41</c:f>
               <c:strCache>
-                <c:ptCount val="46"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>Jul 2022</c:v>
+                  <c:v>Jan 2023</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Aug 2022</c:v>
+                  <c:v>Feb 2023</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sep 2022</c:v>
+                  <c:v>Mar 2023</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Oct 2022</c:v>
+                  <c:v>Apr 2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Nov 2022</c:v>
+                  <c:v>May 2023</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Dec 2022</c:v>
+                  <c:v>Jun 2023</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Jan 2023</c:v>
+                  <c:v>Jul 2023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Feb 2023</c:v>
+                  <c:v>Aug 2023</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Mar 2023</c:v>
+                  <c:v>Sep 2023</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Apr 2023</c:v>
+                  <c:v>Oct 2023</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>May 2023</c:v>
+                  <c:v>Nov 2023</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Jun 2023</c:v>
+                  <c:v>Dec 2023</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Jul 2023</c:v>
+                  <c:v>Jan 2024</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Aug 2023</c:v>
+                  <c:v>Feb 2024</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Sep 2023</c:v>
+                  <c:v>Mar 2024</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>Oct 2023</c:v>
+                  <c:v>Apr 2024</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Nov 2023</c:v>
+                  <c:v>May 2024</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>Dec 2023</c:v>
+                  <c:v>Jun 2024</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>Jan 2024</c:v>
+                  <c:v>Jul 2024</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>Feb 2024</c:v>
+                  <c:v>Aug 2024</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>Mar 2024</c:v>
+                  <c:v>Sep 2024</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>Apr 2024</c:v>
+                  <c:v>Oct 2024</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>May 2024</c:v>
+                  <c:v>Nov 2024</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>Jun 2024</c:v>
+                  <c:v>Dec 2024</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>Jul 2024</c:v>
+                  <c:v>Jan 2025</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>Aug 2024</c:v>
+                  <c:v>Feb 2025</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>Sep 2024</c:v>
+                  <c:v>Mar 2025</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>Oct 2024</c:v>
+                  <c:v>Apr 2025</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>Nov 2024</c:v>
+                  <c:v>May 2025</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>Dec 2024</c:v>
+                  <c:v>Jun 2025</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>Jan 2025</c:v>
+                  <c:v>Jul 2025</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>Feb 2025</c:v>
+                  <c:v>Aug 2025</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>Mar 2025</c:v>
+                  <c:v>Sep 2025</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>Apr 2025</c:v>
+                  <c:v>Oct 2025</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>May 2025</c:v>
+                  <c:v>Nov 2025</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>Jun 2025</c:v>
+                  <c:v>Dec 2025</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>Jul 2025</c:v>
+                  <c:v>Jan 2026</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>Aug 2025</c:v>
+                  <c:v>Feb 2026</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>Sep 2025</c:v>
+                  <c:v>Mar 2026</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>Oct 2025</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>Nov 2025</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>Dec 2025</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>Jan 2026</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>Feb 2026</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>Mar 2026</c:v>
-                </c:pt>
-                <c:pt idx="45">
                   <c:v>Apr 2026</c:v>
                 </c:pt>
               </c:strCache>
@@ -1658,146 +1540,128 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$E$2:$E$47</c:f>
+              <c:f>Data!$E$2:$E$41</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="46"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>5.74</c:v>
+                  <c:v>1.01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.29</c:v>
+                  <c:v>1.08</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2.23</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.57</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.31</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.64</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.49</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.04</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.66</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.12</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.8</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.38</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.02</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.98</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.12</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.47</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8.98</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.14</c:v>
+                </c:pt>
+                <c:pt idx="18">
                   <c:v>2.62</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>2.7</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.66</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.12</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.01</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.08</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2.23</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2.46</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>4.31</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.64</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.49</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>2.04</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.96</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.26</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>1.8</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0.89</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>2.02</c:v>
-                </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.24</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1.12</c:v>
+                  <c:v>1.53</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1.47</c:v>
+                  <c:v>1.94</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>8.98</c:v>
+                  <c:v>7.41</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.16</c:v>
+                  <c:v>3.69</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.24</c:v>
+                  <c:v>2.08</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>2.58</c:v>
+                  <c:v>1.77</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.35</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1.94</c:v>
+                  <c:v>2.07</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>4.99</c:v>
+                  <c:v>2.9</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1.22</c:v>
+                  <c:v>7.74</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.24</c:v>
+                  <c:v>1.57</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.6</c:v>
+                  <c:v>1.81</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>1.9</c:v>
+                  <c:v>1.46</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.98</c:v>
+                  <c:v>1.76</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>1.48</c:v>
+                  <c:v>2.33</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>4.24</c:v>
+                  <c:v>1.83</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.1</c:v>
+                  <c:v>1.54</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>2.41</c:v>
+                  <c:v>1.44</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>1.46</c:v>
+                  <c:v>0.65</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>1.76</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>-0.54</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>0.38</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>1.54</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>1.46</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>0.65</c:v>
-                </c:pt>
-                <c:pt idx="45">
                   <c:v>0.6899999999999999</c:v>
                 </c:pt>
               </c:numCache>
@@ -1829,145 +1693,127 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$J$2:$J$47</c:f>
+              <c:f>Data!$J$2:$J$41</c:f>
               <c:strCache>
-                <c:ptCount val="46"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>Jul 2022</c:v>
+                  <c:v>Jan 2023</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Aug 2022</c:v>
+                  <c:v>Feb 2023</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sep 2022</c:v>
+                  <c:v>Mar 2023</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Oct 2022</c:v>
+                  <c:v>Apr 2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Nov 2022</c:v>
+                  <c:v>May 2023</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Dec 2022</c:v>
+                  <c:v>Jun 2023</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Jan 2023</c:v>
+                  <c:v>Jul 2023</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Feb 2023</c:v>
+                  <c:v>Aug 2023</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Mar 2023</c:v>
+                  <c:v>Sep 2023</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Apr 2023</c:v>
+                  <c:v>Oct 2023</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>May 2023</c:v>
+                  <c:v>Nov 2023</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Jun 2023</c:v>
+                  <c:v>Dec 2023</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>Jul 2023</c:v>
+                  <c:v>Jan 2024</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Aug 2023</c:v>
+                  <c:v>Feb 2024</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>Sep 2023</c:v>
+                  <c:v>Mar 2024</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>Oct 2023</c:v>
+                  <c:v>Apr 2024</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>Nov 2023</c:v>
+                  <c:v>May 2024</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>Dec 2023</c:v>
+                  <c:v>Jun 2024</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>Jan 2024</c:v>
+                  <c:v>Jul 2024</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>Feb 2024</c:v>
+                  <c:v>Aug 2024</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>Mar 2024</c:v>
+                  <c:v>Sep 2024</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>Apr 2024</c:v>
+                  <c:v>Oct 2024</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>May 2024</c:v>
+                  <c:v>Nov 2024</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>Jun 2024</c:v>
+                  <c:v>Dec 2024</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>Jul 2024</c:v>
+                  <c:v>Jan 2025</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>Aug 2024</c:v>
+                  <c:v>Feb 2025</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>Sep 2024</c:v>
+                  <c:v>Mar 2025</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>Oct 2024</c:v>
+                  <c:v>Apr 2025</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>Nov 2024</c:v>
+                  <c:v>May 2025</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>Dec 2024</c:v>
+                  <c:v>Jun 2025</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>Jan 2025</c:v>
+                  <c:v>Jul 2025</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>Feb 2025</c:v>
+                  <c:v>Aug 2025</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>Mar 2025</c:v>
+                  <c:v>Sep 2025</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>Apr 2025</c:v>
+                  <c:v>Oct 2025</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>May 2025</c:v>
+                  <c:v>Nov 2025</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>Jun 2025</c:v>
+                  <c:v>Dec 2025</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>Jul 2025</c:v>
+                  <c:v>Jan 2026</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>Aug 2025</c:v>
+                  <c:v>Feb 2026</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>Sep 2025</c:v>
+                  <c:v>Mar 2026</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>Oct 2025</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>Nov 2025</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>Dec 2025</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>Jan 2026</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>Feb 2026</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>Mar 2026</c:v>
-                </c:pt>
-                <c:pt idx="45">
                   <c:v>Apr 2026</c:v>
                 </c:pt>
               </c:strCache>
@@ -1975,146 +1821,128 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$K$2:$K$47</c:f>
+              <c:f>Data!$K$2:$K$41</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="46"/>
+                <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>10.5217</c:v>
+                  <c:v>13.9409</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3.65</c:v>
+                  <c:v>-7.9646</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-10.4518</c:v>
+                  <c:v>0.2623</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.6065</c:v>
+                  <c:v>0.8718</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>14.334</c:v>
+                  <c:v>-5.4883</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-6.1629</c:v>
+                  <c:v>3.1093</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13.9409</c:v>
+                  <c:v>5.5306</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-7.9646</c:v>
+                  <c:v>-4.9229</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.2622</c:v>
+                  <c:v>-3.1517</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.8718</c:v>
+                  <c:v>-3.5797</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-5.4883</c:v>
+                  <c:v>8.244899999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.1093</c:v>
+                  <c:v>8.418699999999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.5306</c:v>
+                  <c:v>-0.9875</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-4.923</c:v>
+                  <c:v>1.2701</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-3.1517</c:v>
+                  <c:v>3.0936</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.5797</c:v>
+                  <c:v>-5.3528</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>8.244899999999999</c:v>
+                  <c:v>5.6127</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.418699999999999</c:v>
+                  <c:v>-0.8925</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-0.9875</c:v>
+                  <c:v>4.3916</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.2701</c:v>
+                  <c:v>3.3973</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3.0936</c:v>
+                  <c:v>4.7932</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-5.3528</c:v>
+                  <c:v>-6.4921</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>5.6127</c:v>
+                  <c:v>4.2604</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-0.8925</c:v>
+                  <c:v>-9.723800000000001</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>4.3916</c:v>
+                  <c:v>4.8823</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>3.3973</c:v>
+                  <c:v>-2.5193</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>4.7932</c:v>
+                  <c:v>-2.2926</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-6.4921</c:v>
+                  <c:v>5.2474</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>4.2604</c:v>
+                  <c:v>4.621</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-9.723800000000001</c:v>
+                  <c:v>1.976</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>4.8823</c:v>
+                  <c:v>0.3742</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-2.5193</c:v>
+                  <c:v>4.0738</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-2.2926</c:v>
+                  <c:v>-0.2954</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>5.2474</c:v>
+                  <c:v>-0.8519</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>4.621</c:v>
+                  <c:v>-3.4367</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>1.976</c:v>
+                  <c:v>1.3153</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.3742</c:v>
+                  <c:v>7.7676</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>4.0738</c:v>
+                  <c:v>8.432399999999999</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-0.2954</c:v>
+                  <c:v>-7.7434</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-0.8519</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>-3.4367</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>1.3153</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>7.7676</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>8.432399999999999</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>-7.7434</c:v>
-                </c:pt>
-                <c:pt idx="45">
                   <c:v>6.232</c:v>
                 </c:pt>
               </c:numCache>
@@ -2663,7 +2491,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q63"/>
+  <dimension ref="A1:Q62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.42578125" customWidth="1"/>
@@ -2676,7 +2504,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="14" customHeight="1">
       <c r="B1" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2695,7 +2523,7 @@
     </row>
     <row r="2" spans="1:17" ht="26" customHeight="1">
       <c r="B2" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2714,7 +2542,7 @@
     </row>
     <row r="3" spans="1:17" ht="26" customHeight="1">
       <c r="B3" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2753,7 +2581,7 @@
     <row r="5" spans="1:17" ht="8" customHeight="1"/>
     <row r="6" spans="1:17" ht="17" customHeight="1">
       <c r="B6" s="5" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2763,7 +2591,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -2774,7 +2602,7 @@
     </row>
     <row r="7" spans="1:17">
       <c r="B7" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2784,7 +2612,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
@@ -2795,7 +2623,7 @@
     </row>
     <row r="8" spans="1:17">
       <c r="B8" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -2814,7 +2642,7 @@
     </row>
     <row r="9" spans="1:17">
       <c r="B9" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -2833,7 +2661,7 @@
     </row>
     <row r="10" spans="1:17">
       <c r="B10" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -2852,7 +2680,7 @@
     </row>
     <row r="11" spans="1:17">
       <c r="B11" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -2888,7 +2716,7 @@
     </row>
     <row r="13" spans="1:17" ht="17" customHeight="1">
       <c r="B13" s="5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -2898,7 +2726,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
@@ -2909,7 +2737,7 @@
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
       <c r="B14" s="7" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -2919,14 +2747,14 @@
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="8" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
       <c r="O14" s="8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="P14" s="8"/>
     </row>
@@ -2940,20 +2768,20 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="9" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
       <c r="N15" s="9"/>
       <c r="O15" s="9" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="P15" s="9"/>
     </row>
     <row r="16" spans="1:17" ht="12" customHeight="1">
       <c r="B16" s="10" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -2963,20 +2791,20 @@
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
       <c r="J16" s="8" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
       <c r="O16" s="8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="P16" s="8"/>
     </row>
     <row r="17" spans="2:16" ht="18" customHeight="1">
       <c r="B17" s="10" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -2986,20 +2814,20 @@
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
       <c r="J17" s="9" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="K17" s="9"/>
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="9"/>
       <c r="O17" s="9" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="P17" s="9"/>
     </row>
     <row r="18" spans="2:16" ht="10" customHeight="1">
       <c r="B18" s="10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
@@ -3018,7 +2846,7 @@
     </row>
     <row r="19" spans="2:16" ht="17" customHeight="1">
       <c r="B19" s="10" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
@@ -3028,7 +2856,7 @@
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
       <c r="J19" s="5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
@@ -3039,7 +2867,7 @@
     </row>
     <row r="20" spans="2:16">
       <c r="B20" s="10" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -3049,14 +2877,14 @@
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
       <c r="J20" s="11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="K20" s="11"/>
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
       <c r="O20" s="12" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="P20" s="12"/>
     </row>
@@ -3070,20 +2898,20 @@
       <c r="H21" s="10"/>
       <c r="I21" s="10"/>
       <c r="J21" s="11" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="K21" s="11"/>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
       <c r="N21" s="11"/>
       <c r="O21" s="12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="P21" s="12"/>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" s="10" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -3093,20 +2921,20 @@
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
       <c r="J22" s="11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="K22" s="11"/>
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
       <c r="N22" s="11"/>
       <c r="O22" s="12" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="P22" s="12"/>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" s="10" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
@@ -3116,14 +2944,14 @@
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
       <c r="J23" s="11" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K23" s="11"/>
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
       <c r="N23" s="11"/>
       <c r="O23" s="12" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="P23" s="12"/>
     </row>
@@ -3137,14 +2965,14 @@
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
       <c r="J24" s="11" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="K24" s="11"/>
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
       <c r="N24" s="11"/>
       <c r="O24" s="12" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="P24" s="12"/>
     </row>
@@ -3167,7 +2995,7 @@
     </row>
     <row r="26" spans="2:16" ht="17" customHeight="1">
       <c r="B26" s="5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -3177,7 +3005,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
@@ -3196,14 +3024,14 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="11" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="K27" s="11"/>
       <c r="L27" s="11"/>
       <c r="M27" s="11"/>
       <c r="N27" s="11"/>
       <c r="O27" s="13" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="P27" s="13"/>
     </row>
@@ -3217,14 +3045,14 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="11" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="K28" s="11"/>
       <c r="L28" s="11"/>
       <c r="M28" s="11"/>
       <c r="N28" s="11"/>
       <c r="O28" s="13" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="P28" s="13"/>
     </row>
@@ -3238,14 +3066,14 @@
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="K29" s="11"/>
       <c r="L29" s="11"/>
       <c r="M29" s="11"/>
       <c r="N29" s="11"/>
       <c r="O29" s="13" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="P29" s="13"/>
     </row>
@@ -3259,14 +3087,14 @@
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="K30" s="11"/>
       <c r="L30" s="11"/>
       <c r="M30" s="11"/>
       <c r="N30" s="11"/>
       <c r="O30" s="13" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="P30" s="13"/>
     </row>
@@ -3426,7 +3254,7 @@
     <row r="40" spans="2:16" ht="10" customHeight="1"/>
     <row r="41" spans="2:16" ht="17" customHeight="1">
       <c r="B41" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -3633,7 +3461,7 @@
     <row r="53" spans="2:16" ht="8" customHeight="1"/>
     <row r="54" spans="2:16" ht="17" customHeight="1">
       <c r="B54" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
@@ -3653,46 +3481,46 @@
     <row r="55" spans="2:16" ht="16" customHeight="1">
       <c r="B55" s="14"/>
       <c r="C55" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D55" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H55" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="I55" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="D55" s="14" t="s">
+      <c r="J55" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="E55" s="14" t="s">
+      <c r="K55" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="F55" s="14" t="s">
+      <c r="L55" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="G55" s="14" t="s">
+      <c r="M55" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="H55" s="14" t="s">
+      <c r="N55" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="I55" s="14" t="s">
+      <c r="O55" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="J55" s="14" t="s">
+      <c r="P55" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="K55" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="L55" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="M55" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="N55" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="O55" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="P55" s="14" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="56" spans="2:16" ht="14" customHeight="1">
@@ -3703,7 +3531,7 @@
         <v>1.54</v>
       </c>
       <c r="D56" s="16">
-        <v>1.46</v>
+        <v>1.44</v>
       </c>
       <c r="E56" s="16">
         <v>0.65</v>
@@ -3720,7 +3548,7 @@
       <c r="M56" s="17"/>
       <c r="N56" s="17"/>
       <c r="O56" s="18">
-        <v>4.41</v>
+        <v>4.39</v>
       </c>
       <c r="P56" s="16">
         <v>14.52</v>
@@ -3731,28 +3559,28 @@
         <v>2025</v>
       </c>
       <c r="C57" s="20">
-        <v>0.24</v>
+        <v>2.08</v>
       </c>
       <c r="D57" s="20">
-        <v>0.6</v>
+        <v>1.77</v>
       </c>
       <c r="E57" s="20">
         <v>1.9</v>
       </c>
       <c r="F57" s="20">
-        <v>0.98</v>
+        <v>2.07</v>
       </c>
       <c r="G57" s="20">
-        <v>1.48</v>
+        <v>2.9</v>
       </c>
       <c r="H57" s="20">
-        <v>4.24</v>
+        <v>7.74</v>
       </c>
       <c r="I57" s="20">
-        <v>0.1</v>
+        <v>1.57</v>
       </c>
       <c r="J57" s="20">
-        <v>2.41</v>
+        <v>1.81</v>
       </c>
       <c r="K57" s="20">
         <v>1.46</v>
@@ -3760,14 +3588,14 @@
       <c r="L57" s="20">
         <v>1.76</v>
       </c>
-      <c r="M57" s="21">
-        <v>-0.54</v>
+      <c r="M57" s="20">
+        <v>2.33</v>
       </c>
       <c r="N57" s="20">
-        <v>0.38</v>
-      </c>
-      <c r="O57" s="22">
-        <v>15.99</v>
+        <v>1.83</v>
+      </c>
+      <c r="O57" s="21">
+        <v>33.27</v>
       </c>
       <c r="P57" s="20">
         <v>13.33</v>
@@ -3781,7 +3609,7 @@
         <v>2.02</v>
       </c>
       <c r="D58" s="16">
-        <v>1.24</v>
+        <v>2.98</v>
       </c>
       <c r="E58" s="16">
         <v>1.12</v>
@@ -3793,28 +3621,28 @@
         <v>8.98</v>
       </c>
       <c r="H58" s="16">
-        <v>1.16</v>
+        <v>2.14</v>
       </c>
       <c r="I58" s="16">
-        <v>0.24</v>
+        <v>2.62</v>
       </c>
       <c r="J58" s="16">
-        <v>2.58</v>
+        <v>5.5</v>
       </c>
       <c r="K58" s="16">
-        <v>0.35</v>
+        <v>1.53</v>
       </c>
       <c r="L58" s="16">
         <v>1.94</v>
       </c>
       <c r="M58" s="16">
-        <v>4.99</v>
+        <v>7.41</v>
       </c>
       <c r="N58" s="16">
-        <v>1.22</v>
+        <v>3.69</v>
       </c>
       <c r="O58" s="18">
-        <v>30.6</v>
+        <v>49.75</v>
       </c>
       <c r="P58" s="16">
         <v>1.95</v>
@@ -3834,7 +3662,7 @@
         <v>2.23</v>
       </c>
       <c r="F59" s="20">
-        <v>2.46</v>
+        <v>1.57</v>
       </c>
       <c r="G59" s="20">
         <v>4.31</v>
@@ -3849,97 +3677,62 @@
         <v>2.04</v>
       </c>
       <c r="K59" s="20">
-        <v>0.96</v>
+        <v>1.66</v>
       </c>
       <c r="L59" s="20">
-        <v>0.26</v>
+        <v>1.12</v>
       </c>
       <c r="M59" s="20">
         <v>1.8</v>
       </c>
       <c r="N59" s="20">
-        <v>0.89</v>
-      </c>
-      <c r="O59" s="22">
-        <v>22.07</v>
+        <v>1.38</v>
+      </c>
+      <c r="O59" s="21">
+        <v>23.49</v>
       </c>
       <c r="P59" s="20">
         <v>13.65</v>
       </c>
     </row>
-    <row r="60" spans="2:16" ht="14" customHeight="1">
-      <c r="B60" s="15">
-        <v>2022</v>
-      </c>
-      <c r="C60" s="17"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-      <c r="H60" s="17"/>
-      <c r="I60" s="16">
-        <v>5.74</v>
-      </c>
-      <c r="J60" s="16">
-        <v>3.29</v>
-      </c>
-      <c r="K60" s="16">
-        <v>2.62</v>
-      </c>
-      <c r="L60" s="16">
-        <v>2.7</v>
-      </c>
-      <c r="M60" s="16">
-        <v>1.66</v>
-      </c>
-      <c r="N60" s="16">
-        <v>1.12</v>
-      </c>
-      <c r="O60" s="18">
-        <v>18.33</v>
-      </c>
-      <c r="P60" s="16">
-        <v>8.039999999999999</v>
-      </c>
-    </row>
-    <row r="61" spans="2:16" ht="6" customHeight="1"/>
-    <row r="62" spans="2:16" ht="40" customHeight="1">
-      <c r="B62" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="C62" s="23"/>
-      <c r="D62" s="23"/>
-      <c r="E62" s="23"/>
-      <c r="F62" s="23"/>
-      <c r="G62" s="23"/>
-      <c r="H62" s="23"/>
-      <c r="I62" s="23"/>
-      <c r="J62" s="23"/>
-      <c r="K62" s="23"/>
-      <c r="L62" s="23"/>
-      <c r="M62" s="23"/>
-      <c r="N62" s="23"/>
-      <c r="O62" s="23"/>
-      <c r="P62" s="23"/>
-    </row>
-    <row r="63" spans="2:16" ht="16" customHeight="1">
-      <c r="B63" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
-      <c r="M63" s="10"/>
-      <c r="N63" s="10"/>
-      <c r="O63" s="10"/>
-      <c r="P63" s="10"/>
+    <row r="60" spans="2:16" ht="6" customHeight="1"/>
+    <row r="61" spans="2:16" ht="40" customHeight="1">
+      <c r="B61" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C61" s="22"/>
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="22"/>
+      <c r="H61" s="22"/>
+      <c r="I61" s="22"/>
+      <c r="J61" s="22"/>
+      <c r="K61" s="22"/>
+      <c r="L61" s="22"/>
+      <c r="M61" s="22"/>
+      <c r="N61" s="22"/>
+      <c r="O61" s="22"/>
+      <c r="P61" s="22"/>
+    </row>
+    <row r="62" spans="2:16" ht="16" customHeight="1">
+      <c r="B62" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" s="10"/>
+      <c r="D62" s="10"/>
+      <c r="E62" s="10"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="10"/>
+      <c r="H62" s="10"/>
+      <c r="I62" s="10"/>
+      <c r="J62" s="10"/>
+      <c r="K62" s="10"/>
+      <c r="L62" s="10"/>
+      <c r="M62" s="10"/>
+      <c r="N62" s="10"/>
+      <c r="O62" s="10"/>
+      <c r="P62" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="101">
@@ -4042,8 +3835,8 @@
     <mergeCell ref="B51:P51"/>
     <mergeCell ref="B52:P52"/>
     <mergeCell ref="B54:P54"/>
+    <mergeCell ref="B61:P61"/>
     <mergeCell ref="B62:P62"/>
-    <mergeCell ref="B63:P63"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.45" bottom="0.45" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
@@ -4053,7 +3846,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -4067,19 +3860,19 @@
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G1" t="s">
         <v>0</v>
       </c>
       <c r="H1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
       </c>
       <c r="K1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -4093,7 +3886,7 @@
         <v>2</v>
       </c>
       <c r="E2">
-        <v>5.74</v>
+        <v>1.01</v>
       </c>
       <c r="G2" t="s">
         <v>2</v>
@@ -4105,7 +3898,7 @@
         <v>2</v>
       </c>
       <c r="K2">
-        <v>10.5217</v>
+        <v>13.9409</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -4113,25 +3906,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1057.4</v>
+        <v>1010.1</v>
       </c>
       <c r="D3" t="s">
         <v>3</v>
       </c>
       <c r="E3">
-        <v>3.29</v>
+        <v>1.08</v>
       </c>
       <c r="G3" t="s">
         <v>2</v>
       </c>
       <c r="H3">
-        <v>1105.22</v>
+        <v>1139.41</v>
       </c>
       <c r="J3" t="s">
         <v>3</v>
       </c>
       <c r="K3">
-        <v>-3.65</v>
+        <v>-7.9646</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4139,25 +3932,25 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1092.19</v>
+        <v>1021.01</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4">
-        <v>2.62</v>
+        <v>2.23</v>
       </c>
       <c r="G4" t="s">
         <v>3</v>
       </c>
       <c r="H4">
-        <v>1064.88</v>
+        <v>1048.66</v>
       </c>
       <c r="J4" t="s">
         <v>4</v>
       </c>
       <c r="K4">
-        <v>-10.4518</v>
+        <v>0.2623</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4165,25 +3958,25 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1120.8</v>
+        <v>1043.78</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
       </c>
       <c r="E5">
-        <v>2.7</v>
+        <v>1.57</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
       </c>
       <c r="H5">
-        <v>953.58</v>
+        <v>1051.41</v>
       </c>
       <c r="J5" t="s">
         <v>5</v>
       </c>
       <c r="K5">
-        <v>5.6065</v>
+        <v>0.8718</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4191,25 +3984,25 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1151.07</v>
+        <v>1060.16</v>
       </c>
       <c r="D6" t="s">
         <v>6</v>
       </c>
       <c r="E6">
-        <v>1.66</v>
+        <v>4.31</v>
       </c>
       <c r="G6" t="s">
         <v>5</v>
       </c>
       <c r="H6">
-        <v>1007.04</v>
+        <v>1060.58</v>
       </c>
       <c r="J6" t="s">
         <v>6</v>
       </c>
       <c r="K6">
-        <v>14.334</v>
+        <v>-5.4883</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -4217,25 +4010,25 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1170.17</v>
+        <v>1105.86</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
       </c>
       <c r="E7">
-        <v>1.12</v>
+        <v>1.64</v>
       </c>
       <c r="G7" t="s">
         <v>6</v>
       </c>
       <c r="H7">
-        <v>1151.39</v>
+        <v>1002.37</v>
       </c>
       <c r="J7" t="s">
         <v>7</v>
       </c>
       <c r="K7">
-        <v>-6.1629</v>
+        <v>3.1093</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -4243,25 +4036,25 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1183.28</v>
+        <v>1123.99</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
       </c>
       <c r="E8">
-        <v>1.01</v>
+        <v>1.49</v>
       </c>
       <c r="G8" t="s">
         <v>7</v>
       </c>
       <c r="H8">
-        <v>1080.43</v>
+        <v>1033.53</v>
       </c>
       <c r="J8" t="s">
         <v>8</v>
       </c>
       <c r="K8">
-        <v>13.9409</v>
+        <v>5.5306</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -4269,25 +4062,25 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1195.23</v>
+        <v>1140.74</v>
       </c>
       <c r="D9" t="s">
         <v>9</v>
       </c>
       <c r="E9">
-        <v>1.08</v>
+        <v>2.04</v>
       </c>
       <c r="G9" t="s">
         <v>8</v>
       </c>
       <c r="H9">
-        <v>1231.05</v>
+        <v>1090.7</v>
       </c>
       <c r="J9" t="s">
         <v>9</v>
       </c>
       <c r="K9">
-        <v>-7.9646</v>
+        <v>-4.9229</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -4295,25 +4088,25 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1208.14</v>
+        <v>1164.01</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="E10">
-        <v>2.23</v>
+        <v>1.66</v>
       </c>
       <c r="G10" t="s">
         <v>9</v>
       </c>
       <c r="H10">
-        <v>1133</v>
+        <v>1037</v>
       </c>
       <c r="J10" t="s">
         <v>10</v>
       </c>
       <c r="K10">
-        <v>0.2622</v>
+        <v>-3.1517</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -4321,25 +4114,25 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1235.08</v>
+        <v>1183.34</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11">
-        <v>2.46</v>
+        <v>1.12</v>
       </c>
       <c r="G11" t="s">
         <v>10</v>
       </c>
       <c r="H11">
-        <v>1135.97</v>
+        <v>1004.32</v>
       </c>
       <c r="J11" t="s">
         <v>11</v>
       </c>
       <c r="K11">
-        <v>0.8718</v>
+        <v>-3.5797</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -4347,25 +4140,25 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1265.46</v>
+        <v>1196.59</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12">
-        <v>4.31</v>
+        <v>1.8</v>
       </c>
       <c r="G12" t="s">
         <v>11</v>
       </c>
       <c r="H12">
-        <v>1145.88</v>
+        <v>968.37</v>
       </c>
       <c r="J12" t="s">
         <v>12</v>
       </c>
       <c r="K12">
-        <v>-5.4883</v>
+        <v>8.244899999999999</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -4373,25 +4166,25 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1320</v>
+        <v>1218.13</v>
       </c>
       <c r="D13" t="s">
         <v>13</v>
       </c>
       <c r="E13">
-        <v>1.64</v>
+        <v>1.38</v>
       </c>
       <c r="G13" t="s">
         <v>12</v>
       </c>
       <c r="H13">
-        <v>1082.99</v>
+        <v>1048.21</v>
       </c>
       <c r="J13" t="s">
         <v>13</v>
       </c>
       <c r="K13">
-        <v>3.1093</v>
+        <v>8.418699999999999</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -4399,25 +4192,25 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1341.65</v>
+        <v>1234.94</v>
       </c>
       <c r="D14" t="s">
         <v>14</v>
       </c>
       <c r="E14">
-        <v>1.49</v>
+        <v>2.02</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
       </c>
       <c r="H14">
-        <v>1116.66</v>
+        <v>1136.45</v>
       </c>
       <c r="J14" t="s">
         <v>14</v>
       </c>
       <c r="K14">
-        <v>5.5306</v>
+        <v>-0.9875</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -4425,25 +4218,25 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>1361.64</v>
+        <v>1259.88</v>
       </c>
       <c r="D15" t="s">
         <v>15</v>
       </c>
       <c r="E15">
-        <v>2.04</v>
+        <v>2.98</v>
       </c>
       <c r="G15" t="s">
         <v>14</v>
       </c>
       <c r="H15">
-        <v>1178.42</v>
+        <v>1125.23</v>
       </c>
       <c r="J15" t="s">
         <v>15</v>
       </c>
       <c r="K15">
-        <v>-4.923</v>
+        <v>1.2701</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -4451,25 +4244,25 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>1389.42</v>
+        <v>1297.43</v>
       </c>
       <c r="D16" t="s">
         <v>16</v>
       </c>
       <c r="E16">
-        <v>0.96</v>
+        <v>1.12</v>
       </c>
       <c r="G16" t="s">
         <v>15</v>
       </c>
       <c r="H16">
-        <v>1120.41</v>
+        <v>1139.52</v>
       </c>
       <c r="J16" t="s">
         <v>16</v>
       </c>
       <c r="K16">
-        <v>-3.1517</v>
+        <v>3.0936</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -4477,25 +4270,25 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1402.76</v>
+        <v>1311.96</v>
       </c>
       <c r="D17" t="s">
         <v>17</v>
       </c>
       <c r="E17">
-        <v>0.26</v>
+        <v>1.47</v>
       </c>
       <c r="G17" t="s">
         <v>16</v>
       </c>
       <c r="H17">
-        <v>1085.09</v>
+        <v>1174.77</v>
       </c>
       <c r="J17" t="s">
         <v>17</v>
       </c>
       <c r="K17">
-        <v>-3.5797</v>
+        <v>-5.3528</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -4503,25 +4296,25 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>1406.41</v>
+        <v>1331.24</v>
       </c>
       <c r="D18" t="s">
         <v>18</v>
       </c>
       <c r="E18">
-        <v>1.8</v>
+        <v>8.98</v>
       </c>
       <c r="G18" t="s">
         <v>17</v>
       </c>
       <c r="H18">
-        <v>1046.25</v>
+        <v>1111.89</v>
       </c>
       <c r="J18" t="s">
         <v>18</v>
       </c>
       <c r="K18">
-        <v>8.244899999999999</v>
+        <v>5.6127</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -4529,25 +4322,25 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>1431.72</v>
+        <v>1450.79</v>
       </c>
       <c r="D19" t="s">
         <v>19</v>
       </c>
       <c r="E19">
-        <v>0.89</v>
+        <v>2.14</v>
       </c>
       <c r="G19" t="s">
         <v>18</v>
       </c>
       <c r="H19">
-        <v>1132.51</v>
+        <v>1174.3</v>
       </c>
       <c r="J19" t="s">
         <v>19</v>
       </c>
       <c r="K19">
-        <v>8.418699999999999</v>
+        <v>-0.8925</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -4555,25 +4348,25 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>1444.46</v>
+        <v>1481.84</v>
       </c>
       <c r="D20" t="s">
         <v>20</v>
       </c>
       <c r="E20">
-        <v>2.02</v>
+        <v>2.62</v>
       </c>
       <c r="G20" t="s">
         <v>19</v>
       </c>
       <c r="H20">
-        <v>1227.86</v>
+        <v>1163.82</v>
       </c>
       <c r="J20" t="s">
         <v>20</v>
       </c>
       <c r="K20">
-        <v>-0.9875</v>
+        <v>4.3916</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -4581,25 +4374,25 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>1473.64</v>
+        <v>1520.66</v>
       </c>
       <c r="D21" t="s">
         <v>21</v>
       </c>
       <c r="E21">
-        <v>1.24</v>
+        <v>5.5</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
       </c>
       <c r="H21">
-        <v>1215.73</v>
+        <v>1214.93</v>
       </c>
       <c r="J21" t="s">
         <v>21</v>
       </c>
       <c r="K21">
-        <v>1.2701</v>
+        <v>3.3973</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -4607,25 +4400,25 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>1491.92</v>
+        <v>1604.3</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
       </c>
       <c r="E22">
-        <v>1.12</v>
+        <v>1.53</v>
       </c>
       <c r="G22" t="s">
         <v>21</v>
       </c>
       <c r="H22">
-        <v>1231.17</v>
+        <v>1256.2</v>
       </c>
       <c r="J22" t="s">
         <v>22</v>
       </c>
       <c r="K22">
-        <v>3.0936</v>
+        <v>4.7932</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -4633,25 +4426,25 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>1508.62</v>
+        <v>1628.84</v>
       </c>
       <c r="D23" t="s">
         <v>23</v>
       </c>
       <c r="E23">
-        <v>1.47</v>
+        <v>1.94</v>
       </c>
       <c r="G23" t="s">
         <v>22</v>
       </c>
       <c r="H23">
-        <v>1269.26</v>
+        <v>1316.41</v>
       </c>
       <c r="J23" t="s">
         <v>23</v>
       </c>
       <c r="K23">
-        <v>-5.3528</v>
+        <v>-6.4921</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -4659,25 +4452,25 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>1530.8</v>
+        <v>1660.44</v>
       </c>
       <c r="D24" t="s">
         <v>24</v>
       </c>
       <c r="E24">
-        <v>8.98</v>
+        <v>7.41</v>
       </c>
       <c r="G24" t="s">
         <v>23</v>
       </c>
       <c r="H24">
-        <v>1201.32</v>
+        <v>1230.95</v>
       </c>
       <c r="J24" t="s">
         <v>24</v>
       </c>
       <c r="K24">
-        <v>5.6127</v>
+        <v>4.2604</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -4685,25 +4478,25 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>1668.27</v>
+        <v>1783.48</v>
       </c>
       <c r="D25" t="s">
         <v>25</v>
       </c>
       <c r="E25">
-        <v>1.16</v>
+        <v>3.69</v>
       </c>
       <c r="G25" t="s">
         <v>24</v>
       </c>
       <c r="H25">
-        <v>1268.75</v>
+        <v>1283.39</v>
       </c>
       <c r="J25" t="s">
         <v>25</v>
       </c>
       <c r="K25">
-        <v>-0.8925</v>
+        <v>-9.723800000000001</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -4711,25 +4504,25 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>1687.62</v>
+        <v>1849.29</v>
       </c>
       <c r="D26" t="s">
         <v>26</v>
       </c>
       <c r="E26">
-        <v>0.24</v>
+        <v>2.08</v>
       </c>
       <c r="G26" t="s">
         <v>25</v>
       </c>
       <c r="H26">
-        <v>1257.42</v>
+        <v>1158.6</v>
       </c>
       <c r="J26" t="s">
         <v>26</v>
       </c>
       <c r="K26">
-        <v>4.3916</v>
+        <v>4.8823</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -4737,25 +4530,25 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>1691.67</v>
+        <v>1887.76</v>
       </c>
       <c r="D27" t="s">
         <v>27</v>
       </c>
       <c r="E27">
-        <v>2.58</v>
+        <v>1.77</v>
       </c>
       <c r="G27" t="s">
         <v>26</v>
       </c>
       <c r="H27">
-        <v>1312.64</v>
+        <v>1215.17</v>
       </c>
       <c r="J27" t="s">
         <v>27</v>
       </c>
       <c r="K27">
-        <v>3.3973</v>
+        <v>-2.5193</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -4763,25 +4556,25 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>1735.31</v>
+        <v>1921.17</v>
       </c>
       <c r="D28" t="s">
         <v>28</v>
       </c>
       <c r="E28">
-        <v>0.35</v>
+        <v>1.9</v>
       </c>
       <c r="G28" t="s">
         <v>27</v>
       </c>
       <c r="H28">
-        <v>1357.24</v>
+        <v>1184.55</v>
       </c>
       <c r="J28" t="s">
         <v>28</v>
       </c>
       <c r="K28">
-        <v>4.7932</v>
+        <v>-2.2926</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -4789,25 +4582,25 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>1741.39</v>
+        <v>1957.67</v>
       </c>
       <c r="D29" t="s">
         <v>29</v>
       </c>
       <c r="E29">
-        <v>1.94</v>
+        <v>2.07</v>
       </c>
       <c r="G29" t="s">
         <v>28</v>
       </c>
       <c r="H29">
-        <v>1422.29</v>
+        <v>1157.4</v>
       </c>
       <c r="J29" t="s">
         <v>29</v>
       </c>
       <c r="K29">
-        <v>-6.4921</v>
+        <v>5.2474</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -4815,25 +4608,25 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>1775.17</v>
+        <v>1998.2</v>
       </c>
       <c r="D30" t="s">
         <v>30</v>
       </c>
       <c r="E30">
-        <v>4.99</v>
+        <v>2.9</v>
       </c>
       <c r="G30" t="s">
         <v>29</v>
       </c>
       <c r="H30">
-        <v>1329.96</v>
+        <v>1218.13</v>
       </c>
       <c r="J30" t="s">
         <v>30</v>
       </c>
       <c r="K30">
-        <v>4.2604</v>
+        <v>4.621</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -4841,25 +4634,25 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>1863.75</v>
+        <v>2056.14</v>
       </c>
       <c r="D31" t="s">
         <v>31</v>
       </c>
       <c r="E31">
-        <v>1.22</v>
+        <v>7.74</v>
       </c>
       <c r="G31" t="s">
         <v>30</v>
       </c>
       <c r="H31">
-        <v>1386.62</v>
+        <v>1274.42</v>
       </c>
       <c r="J31" t="s">
         <v>31</v>
       </c>
       <c r="K31">
-        <v>-9.723800000000001</v>
+        <v>1.976</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -4867,25 +4660,25 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>1886.49</v>
+        <v>2215.29</v>
       </c>
       <c r="D32" t="s">
         <v>32</v>
       </c>
       <c r="E32">
-        <v>0.24</v>
+        <v>1.57</v>
       </c>
       <c r="G32" t="s">
         <v>31</v>
       </c>
       <c r="H32">
-        <v>1251.79</v>
+        <v>1299.6</v>
       </c>
       <c r="J32" t="s">
         <v>32</v>
       </c>
       <c r="K32">
-        <v>4.8823</v>
+        <v>0.3742</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -4893,25 +4686,25 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>1891.02</v>
+        <v>2250.07</v>
       </c>
       <c r="D33" t="s">
         <v>33</v>
       </c>
       <c r="E33">
-        <v>0.6</v>
+        <v>1.81</v>
       </c>
       <c r="G33" t="s">
         <v>32</v>
       </c>
       <c r="H33">
-        <v>1312.9</v>
+        <v>1304.46</v>
       </c>
       <c r="J33" t="s">
         <v>33</v>
       </c>
       <c r="K33">
-        <v>-2.5193</v>
+        <v>4.0738</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -4919,25 +4712,25 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>1902.36</v>
+        <v>2290.8</v>
       </c>
       <c r="D34" t="s">
         <v>34</v>
       </c>
       <c r="E34">
-        <v>1.9</v>
+        <v>1.46</v>
       </c>
       <c r="G34" t="s">
         <v>33</v>
       </c>
       <c r="H34">
-        <v>1279.83</v>
+        <v>1357.61</v>
       </c>
       <c r="J34" t="s">
         <v>34</v>
       </c>
       <c r="K34">
-        <v>-2.2926</v>
+        <v>-0.2954</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -4945,25 +4738,25 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>1938.51</v>
+        <v>2324.24</v>
       </c>
       <c r="D35" t="s">
         <v>35</v>
       </c>
       <c r="E35">
-        <v>0.98</v>
+        <v>1.76</v>
       </c>
       <c r="G35" t="s">
         <v>34</v>
       </c>
       <c r="H35">
-        <v>1250.48</v>
+        <v>1353.59</v>
       </c>
       <c r="J35" t="s">
         <v>35</v>
       </c>
       <c r="K35">
-        <v>5.2474</v>
+        <v>-0.8519</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -4971,25 +4764,25 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>1957.51</v>
+        <v>2365.15</v>
       </c>
       <c r="D36" t="s">
         <v>36</v>
       </c>
       <c r="E36">
-        <v>1.48</v>
+        <v>2.33</v>
       </c>
       <c r="G36" t="s">
         <v>35</v>
       </c>
       <c r="H36">
-        <v>1316.1</v>
+        <v>1342.06</v>
       </c>
       <c r="J36" t="s">
         <v>36</v>
       </c>
       <c r="K36">
-        <v>4.621</v>
+        <v>-3.4367</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -4997,25 +4790,25 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>1986.48</v>
+        <v>2420.26</v>
       </c>
       <c r="D37" t="s">
         <v>37</v>
       </c>
       <c r="E37">
-        <v>4.24</v>
+        <v>1.83</v>
       </c>
       <c r="G37" t="s">
         <v>36</v>
       </c>
       <c r="H37">
-        <v>1376.92</v>
+        <v>1295.94</v>
       </c>
       <c r="J37" t="s">
         <v>37</v>
       </c>
       <c r="K37">
-        <v>1.976</v>
+        <v>1.3153</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -5023,25 +4816,25 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>2070.7</v>
+        <v>2464.55</v>
       </c>
       <c r="D38" t="s">
         <v>38</v>
       </c>
       <c r="E38">
-        <v>0.1</v>
+        <v>1.54</v>
       </c>
       <c r="G38" t="s">
         <v>37</v>
       </c>
       <c r="H38">
-        <v>1404.13</v>
+        <v>1312.99</v>
       </c>
       <c r="J38" t="s">
         <v>38</v>
       </c>
       <c r="K38">
-        <v>0.3742</v>
+        <v>7.7676</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -5049,25 +4842,25 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>2072.77</v>
+        <v>2502.5</v>
       </c>
       <c r="D39" t="s">
         <v>39</v>
       </c>
       <c r="E39">
-        <v>2.41</v>
+        <v>1.44</v>
       </c>
       <c r="G39" t="s">
         <v>38</v>
       </c>
       <c r="H39">
-        <v>1409.38</v>
+        <v>1414.97</v>
       </c>
       <c r="J39" t="s">
         <v>39</v>
       </c>
       <c r="K39">
-        <v>4.0738</v>
+        <v>8.432399999999999</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -5075,25 +4868,25 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>2122.73</v>
+        <v>2538.54</v>
       </c>
       <c r="D40" t="s">
         <v>40</v>
       </c>
       <c r="E40">
-        <v>1.46</v>
+        <v>0.65</v>
       </c>
       <c r="G40" t="s">
         <v>39</v>
       </c>
       <c r="H40">
-        <v>1466.8</v>
+        <v>1534.29</v>
       </c>
       <c r="J40" t="s">
         <v>40</v>
       </c>
       <c r="K40">
-        <v>-0.2954</v>
+        <v>-7.7434</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -5101,25 +4894,25 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>2153.72</v>
+        <v>2555.04</v>
       </c>
       <c r="D41" t="s">
         <v>41</v>
       </c>
       <c r="E41">
-        <v>1.76</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G41" t="s">
         <v>40</v>
       </c>
       <c r="H41">
-        <v>1462.46</v>
+        <v>1415.48</v>
       </c>
       <c r="J41" t="s">
         <v>41</v>
       </c>
       <c r="K41">
-        <v>-0.8519</v>
+        <v>6.232</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -5127,169 +4920,13 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>2191.63</v>
-      </c>
-      <c r="D42" t="s">
-        <v>42</v>
-      </c>
-      <c r="E42">
-        <v>-0.54</v>
+        <v>2572.67</v>
       </c>
       <c r="G42" t="s">
         <v>41</v>
       </c>
       <c r="H42">
-        <v>1450.01</v>
-      </c>
-      <c r="J42" t="s">
-        <v>42</v>
-      </c>
-      <c r="K42">
-        <v>-3.4367</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11">
-      <c r="A43" t="s">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>2179.79</v>
-      </c>
-      <c r="D43" t="s">
-        <v>43</v>
-      </c>
-      <c r="E43">
-        <v>0.38</v>
-      </c>
-      <c r="G43" t="s">
-        <v>42</v>
-      </c>
-      <c r="H43">
-        <v>1400.17</v>
-      </c>
-      <c r="J43" t="s">
-        <v>43</v>
-      </c>
-      <c r="K43">
-        <v>1.3153</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11">
-      <c r="A44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>2188.07</v>
-      </c>
-      <c r="D44" t="s">
-        <v>44</v>
-      </c>
-      <c r="E44">
-        <v>1.54</v>
-      </c>
-      <c r="G44" t="s">
-        <v>43</v>
-      </c>
-      <c r="H44">
-        <v>1418.59</v>
-      </c>
-      <c r="J44" t="s">
-        <v>44</v>
-      </c>
-      <c r="K44">
-        <v>7.7676</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11">
-      <c r="A45" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45">
-        <v>2221.77</v>
-      </c>
-      <c r="D45" t="s">
-        <v>45</v>
-      </c>
-      <c r="E45">
-        <v>1.46</v>
-      </c>
-      <c r="G45" t="s">
-        <v>44</v>
-      </c>
-      <c r="H45">
-        <v>1528.78</v>
-      </c>
-      <c r="J45" t="s">
-        <v>45</v>
-      </c>
-      <c r="K45">
-        <v>8.432399999999999</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11">
-      <c r="A46" t="s">
-        <v>45</v>
-      </c>
-      <c r="B46">
-        <v>2254.21</v>
-      </c>
-      <c r="D46" t="s">
-        <v>46</v>
-      </c>
-      <c r="E46">
-        <v>0.65</v>
-      </c>
-      <c r="G46" t="s">
-        <v>45</v>
-      </c>
-      <c r="H46">
-        <v>1657.69</v>
-      </c>
-      <c r="J46" t="s">
-        <v>46</v>
-      </c>
-      <c r="K46">
-        <v>-7.7434</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11">
-      <c r="A47" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47">
-        <v>2268.86</v>
-      </c>
-      <c r="D47" t="s">
-        <v>47</v>
-      </c>
-      <c r="E47">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="G47" t="s">
-        <v>46</v>
-      </c>
-      <c r="H47">
-        <v>1529.33</v>
-      </c>
-      <c r="J47" t="s">
-        <v>47</v>
-      </c>
-      <c r="K47">
-        <v>6.232</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11">
-      <c r="A48" t="s">
-        <v>47</v>
-      </c>
-      <c r="B48">
-        <v>2284.52</v>
-      </c>
-      <c r="G48" t="s">
-        <v>47</v>
-      </c>
-      <c r="H48">
-        <v>1624.64</v>
+        <v>1503.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>